<commit_message>
feat: deploy posting plan v1 [run ci]
</commit_message>
<xml_diff>
--- a/review_products.xlsx
+++ b/review_products.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="630" yWindow="615" windowWidth="37095" windowHeight="17310" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G158"/>
+  <dimension ref="A1:G174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4498,16 +4498,430 @@
           <t>https://s.shopee.co.th/110OWujz86</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
           <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-modfibxbvymma0.webp</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
           <t>done 2026-07-07 05:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>131</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>ยกโหล Nekko อาหารเปียกแมว 70 กรัม12ซอง</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1BJb9Qw4hN</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mofbqutr8kcu6a.webp</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>฿159</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>132</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>FABLEME —PET BASKET เข่งใส่แมว ตระกร้าที่นอนแมวแบบเข่ง สไตล์มินิมอลง</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3B4fX6y9c8</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mnrcaodqhb0k02.webp</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>฿220</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>133</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4AxCiwxzUR</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mhh7zikraarne4.webp</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>฿210</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>134</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2BC8LHMRmu</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>฿542</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>135</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>[ประกันศูนย์ไทย] Oneisall Pet Grooming Vacuum Kit 8 in 1 ตัดขนแมว เครื่องดูดขนแมว ไดร์เป่าขนสุนัข ขนาด2.5L รุ่น BM1</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3LO5jQQjkG</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0h-mdtub2gcu0oe50.webp</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>฿5212</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>136</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/qgkkpnnSC</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>฿7888</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>137</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>((12ซอง คละรสได้)) Pramy พรามี่ อาหารเปียกแมว หลากหลายรส ขนาด 70g. สูตรลูกแมว แมวโต แมวสูงวัย</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8KmlgcYJ3j</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mob33vjgv0gee0.webp</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>฿265</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>138</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>PANDO Pet Dryer Room PD65 แพนโด้ เครื่องเป่าขน สำหรับสัตว์เลี้ยง รุ่น PD65 ตู้เป่าขน อัตโนม</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6L1hIwoeQ7</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mojgkgp81dsf9b.webp</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>฿9990</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>139</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>ห้องน้ำแมวอัจฉริยะ ห้องน้ําแมวอัตโนมัติสามารถเก็บอุจจาระได้โดยอัตโนมัติตามการขับถ่ายของแมว หลีกเลี่ยงกลิ่นแปลก ๆ และยับย</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/20si8zFjb6</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mkf3obhghekg6a.webp</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>฿3199</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>140</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>กล่องเดินทางสัตว์เลี้ยง กรงหิ้วแมว กรงเดินทาง กล่องใส่สัตว์เลี้ยง กรงเดินทาง กล่องใส่สัตว์เลี้ยง</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/BR3xcUYD6</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0g-mbm7xxs7he1kb4.webp</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>฿973</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>141</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Pramy in Gravy 70g อาหารเปียกแมว แมวโต เกรวี่ 12ซอง สำหรับแมว2เดือนขึ้นไป Petus Kingkaew</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2BC8LIUqJB</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mornhzyf1w5qc6.webp</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>฿256</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>142</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>navipet Smart Pet Dryer (Thai Version) ตู้เป่า ขนสัตว์เลี้ยง 72ลิตร O ZONE ฆ่าเชื้อได้ ประกันศูนย์ไทย</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/LkU9vkgr8</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr"/>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mnqj2jpnw45hd8.webp</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>฿7900</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>143</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>ห้องน้ำแมวใหญ่ SMART CAT LITTER BO</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7VDeh6StVB</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr"/>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-822yl-mhwpnsjh6k1wff.webp</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>฿1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>144</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>ขนมแมวเลีย Me-O มีโอ 11 รสชาติ คละรสได้ 11/20/25/36 ซอง | ขนมแมว อาหารแมวเลีย อาหารเสริมแมว</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1gFrkO6YwY</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr"/>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mnyj1j3uxe6ad5.webp</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>฿109</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>145</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>สเปรย์น้ำหอมระงับกลิ่น แบรนด์พราวพาว สูตรอ่อนโยน สารสกัดจากธรรมชาติ 3 กลิ่น หอมละมุนชื่นใจ</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/17dlKLdcu</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr"/>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m2usz5kign3644.webp</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>฿169</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>146</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>กรงไก่กลางแจ้ง คอกไก่ บ้านไก่ ขนาดใหญ่พิเศษ สำหรับการเลี้ยงสัตว์ปีก กันฝน กรงนกยูงและนกพิราบ โครงสร้างขนาดใหญ่</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9Uyj4mysUr</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr"/>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mkdbuy6rdgjr2e.webp</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>฿1224</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: CATDUMB-style review card + caption grounding rules
- card/: self-contained HTML/CSS renderer (skipped for x-bot)
- review.py: card render with PIL fallback, grounded caption/hook prompts,
  skip rows with invalid image_url, remove placeholder xlsx row
- review.yml: install playwright chromium

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/review_products.xlsx
+++ b/review_products.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="630" yWindow="615" windowWidth="37095" windowHeight="17310" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G174"/>
+  <dimension ref="A1:G173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -522,41 +522,10 @@
       </c>
     </row>
     <row r="2" ht="39.95" customHeight="1">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>วางรายละเอียดสินค้าจาก Shopee ทั้งหมดที่นี่</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>https://s.lazada.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://down-th.img.susercontent.com/xxx.jpg</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>ลด 20%</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="345" customHeight="1">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>RAY-BAN JUSTIN- RB4165F 601/71
 Ray-Ban เรแบนเป็นผู้นำด้านการผลิตแว่นกันแดด และแว่นสายตา ที่ได้ความนิยมมากที่สุดทั่วโลก มีให้เลือกหลากหลายสไตล์ เหมาะกับทุกคน และใส่ได้ทั้งผู้หญิงและผู้ชาย
@@ -570,23 +539,23 @@
 Lens Material: Polycarbonate Standard</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>https://s.shopee.co.th/AUqz80oxUd</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>https://s.lazada.co.th/s.Z6PzJE?c=b&amp;t=p-ijr1Q-svKWG</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>https://down-th.img.susercontent.com/file/th-11134201-7r990-lscec08f21gm73.webp
 https://down-th.img.susercontent.com/file/th-11134201-7r98y-lscec0amysmu78.webp</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">฿5,130
 final price indicator icon
@@ -598,17 +567,17 @@
 </t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>done 2026-05-21 13:15</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="409.5" customHeight="1">
-      <c r="A4" t="n">
+    <row r="3" ht="345" customHeight="1">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Sony BRAVIA 3 ทีวี 55 นิ้ว รุ่น K-55S30 4K Ultra HD Smart TV (Google TV) | 4K HDR Processor X1
 รายละเอียดสินค้า
@@ -628,22 +597,22 @@
 เรียกดูภาพยนตร์และรายการทีวีมากกว่า 400,000 ตอนจากบริการสตรีมมิ่งของคุณทั้งหมดในที่เดียว โดยจัดเป็นหัวข้อและแนวเนื้อหาไว้ตามสิ่งที่คุณสนใจ</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>https://s.shopee.co.th/10zvLKc6Ji</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>https://s.lazada.co.th/s.Z6mEyG?c=a&amp;t=p-i0-s0&amp;sub_id1=W1</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>https://down-th.img.susercontent.com/file/th-11134207-7r98v-lvsn9yh5vql9c5.webp</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">฿20,500
 final price indicator icon
@@ -653,179 +622,204 @@
 </t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>done 2026-06-01 13:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="409.5" customHeight="1">
+      <c r="A4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>F&amp;G วิลล่าแมว Cat Villa บ้านแมว กรงแมว วิลล่าไม้เนื้อแข็งตู้แมว ตู้โชว์ไม้เนื้อแข็ง วิลล่าแมวขนาดใหญ จัดส่งภายใน24ชั่วโม ราคา 1999.00 บาท</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3qKMKMpn2h</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m3ytl0pibu8a95.webp</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>done 2026-06-01 13:07</t>
+          <t>done 2026-06-05 11:42</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>F&amp;G วิลล่าแมว Cat Villa บ้านแมว กรงแมว วิลล่าไม้เนื้อแข็งตู้แมว ตู้โชว์ไม้เนื้อแข็ง วิลล่าแมวขนาดใหญ จัดส่งภายใน24ชั่วโม ราคา 1999.00 บาท</t>
+          <t>Rojeco เครื่องให้อาหารแมวอัตโนมัติ ปุ่มกด WIFI ควบคุมอัจฉริยะ ขนาด 2 ลิตร ราคา 1363.00 บาท</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qKMKMpn2h</t>
+          <t>https://s.shopee.co.th/4AxCixh5W9</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m3ytl0pibu8a95.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-mlbsygs3nf9f31.webp</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>done 2026-06-05 11:42</t>
+          <t>done 2026-06-05 11:58</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rojeco เครื่องให้อาหารแมวอัตโนมัติ ปุ่มกด WIFI ควบคุมอัจฉริยะ ขนาด 2 ลิตร ราคา 1363.00 บาท</t>
+          <t>【พร้อมส่ง】 EGGแผ่นรองฉี่สุนัข ซึมซับไดีดี ต่อต้านแบคทีเรีย แผ่นรองฉี่ ผ้ารองฉี่สุนัข แผ่นรองฉี่แมว แผ่นรองซับ ทรายแมวCOD ราคา 84.00 บาท</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4AxCixh5W9</t>
+          <t>https://s.shopee.co.th/AAEPs0miQH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-mlbsygs3nf9f31.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul3-lgylrzka8duw84.webp</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>done 2026-06-05 11:58</t>
+          <t>done 2026-06-05 22:49</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>【พร้อมส่ง】 EGGแผ่นรองฉี่สุนัข ซึมซับไดีดี ต่อต้านแบคทีเรีย แผ่นรองฉี่ ผ้ารองฉี่สุนัข แผ่นรองฉี่แมว แผ่นรองซับ ทรายแมวCOD ราคา 84.00 บาท</t>
+          <t>4-6L เครื่องให้อาหารสัตว์เลี้ยงอัตโนมัติ รองรับWiFi &amp; APP เครื่องให้อาหาร เครื่องให้อาหารแมวอัตโนมัติ สําหรับสัตว์เลี้ยง ราคา 491.00 บาท</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AAEPs0miQH</t>
+          <t>https://s.shopee.co.th/7KuEUluFn0</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul3-lgylrzka8duw84.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mmmvfucpjm6db4.webp</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>done 2026-06-05 22:49</t>
+          <t>done 2026-06-06 09:29</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4-6L เครื่องให้อาหารสัตว์เลี้ยงอัตโนมัติ รองรับWiFi &amp; APP เครื่องให้อาหาร เครื่องให้อาหารแมวอัตโนมัติ สําหรับสัตว์เลี้ยง ราคา 491.00 บาท</t>
+          <t>[เลือกรสชาติได้] Purina One อาหารแมว 6.6กก ราคา 1149.00 บาท</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7KuEUluFn0</t>
+          <t>https://s.shopee.co.th/2LVib7bsCQ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mmmvfucpjm6db4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823rm-mp2iqoc9yo7jc3.webp</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>done 2026-06-06 09:29</t>
+          <t>done 2026-06-08 07:45</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[เลือกรสชาติได้] Purina One อาหารแมว 6.6กก ราคา 1149.00 บาท</t>
+          <t>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม ราคา 210.00 บาท</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2LVib7bsCQ</t>
+          <t>https://s.shopee.co.th/70HY9gQhNc</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823rm-mp2iqoc9yo7jc3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mhh7zikraarne4.webp</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>done 2026-06-08 07:45</t>
+          <t>done 2026-06-08 12:14</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>11</v>
+        <v>113</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม ราคา 210.00 บาท</t>
+          <t>MOMOVIDA น้ำพุสัตว์เลี้ยงอัตโนมัติ น้ำพุแมวไร้สาย พร้อมแบตเตอรี่ลิเทียมในตัว 2000 mAh ระบบจ่ายน้ำอัตโนมัติ รุ่น PTM-663 ราคา 899.00 บาท</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/70HY9gQhNc</t>
+          <t>https://s.shopee.co.th/2g8cW8DbOy</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mhh7zikraarne4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-moz7gyb43aiz57.webp</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>done 2026-06-08 12:14</t>
+          <t>done 2026-06-09 06:03</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>113</v>
+        <v>44</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MOMOVIDA น้ำพุสัตว์เลี้ยงอัตโนมัติ น้ำพุแมวไร้สาย พร้อมแบตเตอรี่ลิเทียมในตัว 2000 mAh ระบบจ่ายน้ำอัตโนมัติ รุ่น PTM-663 ราคา 899.00 บาท</t>
+          <t>MOMOVIDA CC-2 กระบะทรายแมวขนาดใหญ่แบบปิด ห้องน้ำแมวทรงโดม มีที่ดักทรายด้านบน ขนาด 64cm กระบะทรายแมว ห้องน้ำแมวขนาดใหญ่ ราคา 939.00 บาท</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2g8cW8DbOy</t>
+          <t>https://s.shopee.co.th/40e06Phd83</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-moz7gyb43aiz57.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-moz7lm82gw0104.webp</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -836,46 +830,46 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>44</v>
+        <v>111</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MOMOVIDA CC-2 กระบะทรายแมวขนาดใหญ่แบบปิด ห้องน้ำแมวทรงโดม มีที่ดักทรายด้านบน ขนาด 64cm กระบะทรายแมว ห้องน้ำแมวขนาดใหญ่ ราคา 939.00 บาท</t>
+          <t>Fiproline [1 กล่อง บรรจุ 2 หลอด] ผลิตภัณฑ์กำจัดเห็บหมัด สำหรับสุนัขและแมว ชนิดหยดหลัง ราคา 142.00 บาท</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/40e06Phd83</t>
+          <t>https://s.shopee.co.th/5fmE5dlGnC</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-moz7lm82gw0104.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mh5q39rleaz229.webp</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>done 2026-06-09 06:03</t>
+          <t>done 2026-06-09 06:04</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>111</v>
+        <v>51</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Fiproline [1 กล่อง บรรจุ 2 หลอด] ผลิตภัณฑ์กำจัดเห็บหมัด สำหรับสุนัขและแมว ชนิดหยดหลัง ราคา 142.00 บาท</t>
+          <t>(ส่งฟรี) ใหม่! ชูชู โปรตีนบูสเตอร์ บำรุงแมว รูปแบบซองเลีย 12 แพ็ค (48ชิ้น) รสปลาแมคเคอเรลและปลาทูน่า ราคา 818.00 บาท</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5fmE5dlGnC</t>
+          <t>https://s.shopee.co.th/1Vwf7pqoPx</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mh5q39rleaz229.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-22110-6nnnf0dtlhjv5d.webp</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -886,21 +880,21 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>51</v>
+        <v>8</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>(ส่งฟรี) ใหม่! ชูชู โปรตีนบูสเตอร์ บำรุงแมว รูปแบบซองเลีย 12 แพ็ค (48ชิ้น) รสปลาแมคเคอเรลและปลาทูน่า ราคา 818.00 บาท</t>
+          <t>P&amp;Pกระบะทรายแมวอัตโนมัติ Automatic Cat Toilet ใช้แอพได้ ดีไซน์ใหญ่ รองรับแมวหลายตัว ห้องน้ำแมวอัตโนมัติ ห้องน้ำแมวอัจฉริยะ ราคา 1388.00 บาท</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1Vwf7pqoPx</t>
+          <t>https://s.shopee.co.th/2g8cVsC5gd</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-22110-6nnnf0dtlhjv5d.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-mj9k7j7ecbno98.webp</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -911,71 +905,71 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>P&amp;Pกระบะทรายแมวอัตโนมัติ Automatic Cat Toilet ใช้แอพได้ ดีไซน์ใหญ่ รองรับแมวหลายตัว ห้องน้ำแมวอัตโนมัติ ห้องน้ำแมวอัจฉริยะ ราคา 1388.00 บาท</t>
+          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK V.3 และ CATLINK V.3 Ultra ราคา 13900.00 บาท</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2g8cVsC5gd</t>
+          <t>https://s.shopee.co.th/6AiUgJSwiQ</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-mj9k7j7ecbno98.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0k-mbdr25xh8y299a.webp</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>done 2026-06-09 06:04</t>
+          <t>done 2026-06-10 06:04</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK V.3 และ CATLINK V.3 Ultra ราคา 13900.00 บาท</t>
+          <t>[ สินค้าใหม่ ] PANDO Aero Cat Litter Box Open-top ห้องน้ำแมวอัตโนมัติ ราคา 7790.00 บาท</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6AiUgJSwiQ</t>
+          <t>https://s.shopee.co.th/9AM6FvSZk3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0k-mbdr25xh8y299a.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mp204c6cw3yjf4.webp</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>done 2026-06-10 06:04</t>
+          <t>done 2026-06-10 06:05</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>52</v>
+        <v>112</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[ สินค้าใหม่ ] PANDO Aero Cat Litter Box Open-top ห้องน้ำแมวอัตโนมัติ ราคา 7790.00 บาท</t>
+          <t>Pramy ทรายแมวเต้าหู้ สูตรไร้ฝุ่น จับตัวเป็นก้อนเร็ว จากใยถั่วเหลืองธรรมชาติ มีให้เลือก 11 กลิ่น ราคา 179.00 บาท</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9AM6FvSZk3</t>
+          <t>https://s.shopee.co.th/2LVm7W68lG</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mp204c6cw3yjf4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mp3itazf1s7h48.webp</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -986,21 +980,21 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>112</v>
+        <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Pramy ทรายแมวเต้าหู้ สูตรไร้ฝุ่น จับตัวเป็นก้อนเร็ว จากใยถั่วเหลืองธรรมชาติ มีให้เลือก 11 กลิ่น ราคา 179.00 บาท</t>
+          <t>ROJECO เครื่องให้อาหารสัตว์เลี้ยงอัตโนมัติ WiFi และแอปควบคุมระยะไกล 4 ลิตร สําหรับสัตว์เลี้ยง สุนัข แมว ราคา 1499.00 บาท</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2LVm7W68lG</t>
+          <t>https://s.shopee.co.th/4AxQIeK8cE</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mp3itazf1s7h48.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/cn-11134207-7r98o-lz47ldvzl6cz24.webp</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1011,21 +1005,21 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ROJECO เครื่องให้อาหารสัตว์เลี้ยงอัตโนมัติ WiFi และแอปควบคุมระยะไกล 4 ลิตร สําหรับสัตว์เลี้ยง สุนัข แมว ราคา 1499.00 บาท</t>
+          <t>(ยกลังสุดคุ้ม) CATE Wet Food เคท อาหารเปียกแมว 5 สูตร บำรุงร่างกาย ไม่เติมเกลือ ไม่ทำร้ายไต (ยกลัง 48 ซอง) ราคา 889.00 บาท</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4AxQIeK8cE</t>
+          <t>https://s.shopee.co.th/5ApxUbxyXR</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/cn-11134207-7r98o-lz47ldvzl6cz24.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mowojgfahclpc3.webp</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1036,71 +1030,71 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>(ยกลังสุดคุ้ม) CATE Wet Food เคท อาหารเปียกแมว 5 สูตร บำรุงร่างกาย ไม่เติมเกลือ ไม่ทำร้ายไต (ยกลัง 48 ซอง) ราคา 889.00 บาท</t>
+          <t>💨ไดร์เป่าขนสัตว์เลี้ยง ไดร์ไล่น้ำ 2800W รุ่น PetPro AirMax สำหรับหมาแมวขนยาว เป่าแห้งเร็ว เสียงเบา | Pettail ร้านค้าไทย ราคา 2190.00 บาท</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5ApxUbxyXR</t>
+          <t>https://s.shopee.co.th/1Vwf7nE9zd</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mowojgfahclpc3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mgbswfbyyn7zea.webp</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>done 2026-06-10 06:05</t>
+          <t>done 2026-06-10 11:15</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>💨ไดร์เป่าขนสัตว์เลี้ยง ไดร์ไล่น้ำ 2800W รุ่น PetPro AirMax สำหรับหมาแมวขนยาว เป่าแห้งเร็ว เสียงเบา | Pettail ร้านค้าไทย ราคา 2190.00 บาท</t>
+          <t>navipet Smart Pet Dryer (Thai Version) ตู้เป่า ขนสัตว์เลี้ยง 72ลิตร O ZONE ฆ่าเชื้อได้ ประกันศูนย์ไทย ราคา 7900.00 บาท</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1Vwf7nE9zd</t>
+          <t>https://s.shopee.co.th/6pyBTXqfWJ</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mgbswfbyyn7zea.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mnqj2jpnw45hd8.webp</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>done 2026-06-10 11:15</t>
+          <t>done 2026-06-10 11:16</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>navipet Smart Pet Dryer (Thai Version) ตู้เป่า ขนสัตว์เลี้ยง 72ลิตร O ZONE ฆ่าเชื้อได้ ประกันศูนย์ไทย ราคา 7900.00 บาท</t>
+          <t>[ขายดี]มีโอ อาหารแมว รสปลาทู 20 กก. / Me-O Cat Food Mackerel 20 kg. ราคา 2100.00 บาท</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6pyBTXqfWJ</t>
+          <t>https://s.shopee.co.th/8pjFrDbySs</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mnqj2jpnw45hd8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/7e2729979fedad3aab036da951c9151b.webp</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1111,21 +1105,21 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>[ขายดี]มีโอ อาหารแมว รสปลาทู 20 กก. / Me-O Cat Food Mackerel 20 kg. ราคา 2100.00 บาท</t>
+          <t>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI ราคา 7714.00 บาท</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8pjFrDbySs</t>
+          <t>https://s.shopee.co.th/5L9KAbNLFq</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/7e2729979fedad3aab036da951c9151b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1136,21 +1130,21 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI ราคา 7714.00 บาท</t>
+          <t>Cutepol 7 ห่อ 28ลิตร (8.75 กิโลกรัม) ทรายแมว ทำจากมันสำปะหลังธรรมชาติ ราคา 669.00 บาท</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5L9KAbNLFq</t>
+          <t>https://s.shopee.co.th/6AiUgQhzZM</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/cn-11134207-7ras8-mbz20lufuzvaa8.webp</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1161,71 +1155,71 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Cutepol 7 ห่อ 28ลิตร (8.75 กิโลกรัม) ทรายแมว ทำจากมันสำปะหลังธรรมชาติ ราคา 669.00 บาท</t>
+          <t>กรงแมว กรงสัตว์เลี้ยง กรงกระต่าย พื้นที่อิสระขนาดใหญ่ กรงแมวขนาดใหญ่ ประกอบง่าย ถอดออกได้ กรงแมวราคาถูก ราคา 1199.00 บาท</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6AiUgQhzZM</t>
+          <t>https://s.shopee.co.th/9zvDFT2WG8</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/cn-11134207-7ras8-mbz20lufuzvaa8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m9een47cb8tc12.webp</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>done 2026-06-10 11:16</t>
+          <t>done 2026-06-11 06:14</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>57</v>
+        <v>5</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>กรงแมว กรงสัตว์เลี้ยง กรงกระต่าย พื้นที่อิสระขนาดใหญ่ กรงแมวขนาดใหญ่ ประกอบง่าย ถอดออกได้ กรงแมวราคาถูก ราคา 1199.00 บาท</t>
+          <t>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์ ราคา 547.00 บาท</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9zvDFT2WG8</t>
+          <t>https://s.shopee.co.th/4AxMmSnMyM</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m9een47cb8tc12.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>done 2026-06-11 06:14</t>
+          <t>done 2026-06-11 06:15</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์ ราคา 547.00 บาท</t>
+          <t>[เลือกรสชาติได้] Purina ONE อาหารแมว 10 kg ราคา 1499.00 บาท</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4AxMmSnMyM</t>
+          <t>https://s.shopee.co.th/8ATVXp85zW</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823ok-mp3h99k9jb4c65.webp</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1236,21 +1230,21 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>9</v>
+        <v>116</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>[เลือกรสชาติได้] Purina ONE อาหารแมว 10 kg ราคา 1499.00 บาท</t>
+          <t>( ใช้โค้ด ส่งฟรีได้ ) ทรายแมว ยกกระสอบ 5 ลิตร x 6 ถุง 30ลิตร เพ็ตโตะซัง Pettosan จับตัวเป็นก้อนดี ราคา 279.00 บาท</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8ATVXp85zW</t>
+          <t>https://s.shopee.co.th/7KuS4iMROy</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823ok-mp3h99k9jb4c65.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m5dz0d7fehme5b.webp</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1261,21 +1255,21 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>( ใช้โค้ด ส่งฟรีได้ ) ทรายแมว ยกกระสอบ 5 ลิตร x 6 ถุง 30ลิตร เพ็ตโตะซัง Pettosan จับตัวเป็นก้อนดี ราคา 279.00 บาท</t>
+          <t>[รุ่นใหม่ 2026!] UrPet FlowX น้ำพุแมวไร้สาย ประกันศูนย์ไทย 1 ปี เชื่อมแอปได้ น้ำพุไร้สาย น้ำพุแมว ราคา 1550.00 บาท</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7KuS4iMROy</t>
+          <t>https://s.shopee.co.th/3LOJJGVua3</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m5dz0d7fehme5b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mory2fab8t1pfd.webp</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1286,46 +1280,46 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>[รุ่นใหม่ 2026!] UrPet FlowX น้ำพุแมวไร้สาย ประกันศูนย์ไทย 1 ปี เชื่อมแอปได้ น้ำพุไร้สาย น้ำพุแมว ราคา 1550.00 บาท</t>
+          <t>พร้อมส่ง คอนโดแมว3ชั้น บ้านแมว หลุมแมว คอนโดแมวหลุมอวกาศ สูง 76ซม. ลับเล็บแมว ฟังก์ชันครบในชิ้นเดียว ราคา 229.00 บาท</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3LOJJGVua3</t>
+          <t>https://s.shopee.co.th/4VaGhLsewN</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mory2fab8t1pfd.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mk279zmozoqte7.webp</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>done 2026-06-11 06:15</t>
+          <t>done 2026-06-12 06:11</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>พร้อมส่ง คอนโดแมว3ชั้น บ้านแมว หลุมแมว คอนโดแมวหลุมอวกาศ สูง 76ซม. ลับเล็บแมว ฟังก์ชันครบในชิ้นเดียว ราคา 229.00 บาท</t>
+          <t>BIO น้ำยาดับกลิ่น กลิ่นฉี่ กลิ่นมูลสัตว์เลี้ยง ล้างพื้นกลิ่นฉี่ ทำความสะอาด ปราศจากเชื้อโรค กลิ่นโอโซนบริสุทธิ์ 1,000 ml ราคา 209.00 บาท</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4VaGhLsewN</t>
+          <t>https://s.shopee.co.th/LkhjkXukD</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mk279zmozoqte7.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-lopnhfgn1k599e.webp</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1336,21 +1330,21 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BIO น้ำยาดับกลิ่น กลิ่นฉี่ กลิ่นมูลสัตว์เลี้ยง ล้างพื้นกลิ่นฉี่ ทำความสะอาด ปราศจากเชื้อโรค กลิ่นโอโซนบริสุทธิ์ 1,000 ml ราคา 209.00 บาท</t>
+          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology ห้องน้ำแมวอัตโนมัติ ปลอดภัยไร้จุดหนีบ CATLINK Baymax ราคา 9900.00 บาท</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/LkhjkXukD</t>
+          <t>https://s.shopee.co.th/9KfWSAow8W</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-lopnhfgn1k599e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0k-mbdr413uxxtta6.webp</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1361,21 +1355,21 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology ห้องน้ำแมวอัตโนมัติ ปลอดภัยไร้จุดหนีบ CATLINK Baymax ราคา 9900.00 บาท</t>
+          <t>【PETStar1】ทรายแมวเต้าหู้ 6L ลิตร.ทรายเต้าหู้ ผลิตจากกากถั่วเหลืองธรรมชาติทราย ละบายกลิ่นได้ดี มีให้เลือก7กลิ่น ราคา 50.00 บาท</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9KfWSAow8W</t>
+          <t>https://s.shopee.co.th/4VaGhPmqmS</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0k-mbdr413uxxtta6.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mep8489kh2pw51.webp</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1386,21 +1380,21 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>【PETStar1】ทรายแมวเต้าหู้ 6L ลิตร.ทรายเต้าหู้ ผลิตจากกากถั่วเหลืองธรรมชาติทราย ละบายกลิ่นได้ดี มีให้เลือก7กลิ่น ราคา 50.00 บาท</t>
+          <t>ลู่วิ่งแมว ออกกำลังกาย ขนาดใหญ่ ที่ออกกำลังกายสัตว์เลี้ยง Pet treadmill ราคา 1062.00 บาท</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4VaGhPmqmS</t>
+          <t>https://s.shopee.co.th/8V6PSay44G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mep8489kh2pw51.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasb-m62hceec0x4m51.webp</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1411,46 +1405,46 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>9</v>
+        <v>69</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ลู่วิ่งแมว ออกกำลังกาย ขนาดใหญ่ ที่ออกกำลังกายสัตว์เลี้ยง Pet treadmill ราคา 1062.00 บาท</t>
+          <t>🔥6L เครื่องให้อาหารอัตโนมัติ🔥 พร้อมกล้องวิดีโอ เครื่องจ่ายอาหารสัตว์เลี้ยง สําหรับสุนัข แมว Smart Pet Feeder Tuya Wifi Camera ราคา 664.00 บาท</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8V6PSay44G</t>
+          <t>https://s.shopee.co.th/8KmzGR87oa</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasb-m62hceec0x4m51.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-7rblj-m5zh8u4bymjb96.webp</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>done 2026-06-12 06:11</t>
+          <t>done 2026-06-13 06:03</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>🔥6L เครื่องให้อาหารอัตโนมัติ🔥 พร้อมกล้องวิดีโอ เครื่องจ่ายอาหารสัตว์เลี้ยง สําหรับสุนัข แมว Smart Pet Feeder Tuya Wifi Camera ราคา 664.00 บาท</t>
+          <t>Lunio Pet Bed ที่นอนสุนัข ที่นอนหมา ที่นอนแมว ที่นอนสัตว์เลี้ยง ทำจากเมมโมรี่โฟม มีคุณสมบัติระบายอากาศได้ดี ราคา 1590.00 บาท</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8KmzGR87oa</t>
+          <t>https://s.shopee.co.th/8KmzGN0nu4</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-7rblj-m5zh8u4bymjb96.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mjtby4ctlkhy74.webp</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1461,21 +1455,21 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Lunio Pet Bed ที่นอนสุนัข ที่นอนหมา ที่นอนแมว ที่นอนสัตว์เลี้ยง ทำจากเมมโมรี่โฟม มีคุณสมบัติระบายอากาศได้ดี ราคา 1590.00 บาท</t>
+          <t>EGGรุ่นใหม่! มีแผ่นกาว แผ่นรองฉี่สุนัข ดูดซับอย่างรวดเร็ว แผ่นรองฉี่ กำจัดกลิ่นดี สุนัข แมว Pet Pad ที่ซับฉี่ COD ราคา 84.00 บาท</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8KmzGN0nu4</t>
+          <t>https://s.shopee.co.th/6pyBTaTs37</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mjtby4ctlkhy74.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mi6pj4eqf1mo06.webp</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1486,21 +1480,21 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>32</v>
+        <v>122</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EGGรุ่นใหม่! มีแผ่นกาว แผ่นรองฉี่สุนัข ดูดซับอย่างรวดเร็ว แผ่นรองฉี่ กำจัดกลิ่นดี สุนัข แมว Pet Pad ที่ซับฉี่ COD ราคา 84.00 บาท</t>
+          <t>Boom Gold Gluten Free บูมโกลด์ กลูเตนฟรี อาหารแมว 15 KG. ราคา 1250.00 บาท</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6pyBTaTs37</t>
+          <t>https://s.shopee.co.th/AKY3eFJHJT</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mi6pj4eqf1mo06.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mp382a0ybxfw09.webp</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1511,71 +1505,71 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>122</v>
+        <v>7</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Boom Gold Gluten Free บูมโกลด์ กลูเตนฟรี อาหารแมว 15 KG. ราคา 1250.00 บาท</t>
+          <t>[ประกันศูนย์ไทย] Oneisall Pet Grooming Vacuum Kit 8 in 1 ตัดขนแมว เครื่องดูดขนแมว ไดร์เป่าขนสุนัข ขนาด2.5L รุ่น BM1 ราคา 5372.00 บาท</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AKY3eFJHJT</t>
+          <t>https://s.shopee.co.th/3qKWNr61yu</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mp382a0ybxfw09.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0h-mdtub2gcu0oe50.webp</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>done 2026-06-13 06:03</t>
+          <t>done 2026-06-13 06:04</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>[ประกันศูนย์ไทย] Oneisall Pet Grooming Vacuum Kit 8 in 1 ตัดขนแมว เครื่องดูดขนแมว ไดร์เป่าขนสุนัข ขนาด2.5L รุ่น BM1 ราคา 5372.00 บาท</t>
+          <t>กรงไก่กลางแจ้ง คอกไก่ บ้านไก่ ขนาดใหญ่พิเศษ สำหรับการเลี้ยงสัตว์ปีก กันฝน กรงนกยูงและนกพิราบ โครงสร้างขนาดใหญ่ ราคา 1186.00 บาท</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qKWNr61yu</t>
+          <t>https://s.shopee.co.th/8Kmvk9b1wJ</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0h-mdtub2gcu0oe50.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mkdbuy6rdgjr2e.webp</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>done 2026-06-13 06:04</t>
+          <t>done 2026-06-14 05:46</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>กรงไก่กลางแจ้ง คอกไก่ บ้านไก่ ขนาดใหญ่พิเศษ สำหรับการเลี้ยงสัตว์ปีก กันฝน กรงนกยูงและนกพิราบ โครงสร้างขนาดใหญ่ ราคา 1186.00 บาท</t>
+          <t>yoyopet : ผ้าเช็ดทำความสะอาดตา หู สัตว์เลี้ยง แบบอ่อนโยน แผ่นเช็ดคราบ สำหรับแมวและสุนัข บรรจุ130ชิ้น ราคา 54.00 บาท</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8Kmvk9b1wJ</t>
+          <t>https://s.shopee.co.th/8ATZ49Q5lO</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mkdbuy6rdgjr2e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m30f7wr2c8er5c.webp</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1586,21 +1580,21 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>yoyopet : ผ้าเช็ดทำความสะอาดตา หู สัตว์เลี้ยง แบบอ่อนโยน แผ่นเช็ดคราบ สำหรับแมวและสุนัข บรรจุ130ชิ้น ราคา 54.00 บาท</t>
+          <t>【พร้อมส่ง】 EGGแผ่นรองฉี่สุนัข ซึมซับไดีดี ต่อต้านแบคทีเรีย แผ่นรองฉี่ ผ้ารองฉี่สุนัข แผ่นรองฉี่แมว แผ่นรองซับ ทรายแมวCOD ราคา 80.00 บาท</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8ATZ49Q5lO</t>
+          <t>https://s.shopee.co.th/2LVm7Rq9pG</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m30f7wr2c8er5c.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul3-lgylrzka8duw84.webp</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1611,46 +1605,46 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>【พร้อมส่ง】 EGGแผ่นรองฉี่สุนัข ซึมซับไดีดี ต่อต้านแบคทีเรีย แผ่นรองฉี่ ผ้ารองฉี่สุนัข แผ่นรองฉี่แมว แผ่นรองซับ ทรายแมวCOD ราคา 80.00 บาท</t>
+          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology น้ำพุแมวที่เก็บสถิติการกินน้ำได้ ฆ่าเชื้อด้วย UV ไส้กรอง UF CATLINK Pure ราคา 2695.00 บาท</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2LVm7Rq9pG</t>
+          <t>https://s.shopee.co.th/gNY8FWitF</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul3-lgylrzka8duw84.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0u-mbdqudvt2aeu73.webp</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>done 2026-06-14 05:46</t>
+          <t>done 2026-06-14 05:47</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology น้ำพุแมวที่เก็บสถิติการกินน้ำได้ ฆ่าเชื้อด้วย UV ไส้กรอง UF CATLINK Pure ราคา 2695.00 บาท</t>
+          <t>แนะนำ! สมาร์ทฮาร์ท โกลด์ ฟิตแอนด์เฟิร์ม 7+ อาหารสุนัขสูงอายุ พันธุ์กลาง-ใหญ่ 20 กก. ราคา 1480.00 บาท</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/gNY8FWitF</t>
+          <t>https://s.shopee.co.th/9pbn350qIc</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0u-mbdqudvt2aeu73.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mp3d3pouixhqeb.webp</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1661,46 +1655,46 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>22</v>
+        <v>123</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>แนะนำ! สมาร์ทฮาร์ท โกลด์ ฟิตแอนด์เฟิร์ม 7+ อาหารสุนัขสูงอายุ พันธุ์กลาง-ใหญ่ 20 กก. ราคา 1480.00 บาท</t>
+          <t>Petcho ที่แปรงขนสัตว์เลี้ยง แปรงขนแมว มีปุ่มดันขนออก ทำความสะอาดง่าย ง่ายต่อการใช้ ราคา 19.00 บาท</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9pbn350qIc</t>
+          <t>https://s.shopee.co.th/70Hbg7eYsX</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mp3d3pouixhqeb.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98w-lyel2mw8dhfla5.webp</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>done 2026-06-14 05:47</t>
+          <t>done 2026-06-15 05:50</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Petcho ที่แปรงขนสัตว์เลี้ยง แปรงขนแมว มีปุ่มดันขนออก ทำความสะอาดง่าย ง่ายต่อการใช้ ราคา 19.00 บาท</t>
+          <t>🔥(120*70CM) แผ่นดักทรายแมว พรมดักทรายแมว พรม 2 ชั้น EVA ช่วยดัก ทรายแมว ที่ติดตามเท้า แผ่น รอง ทรายแมว ขนาด ใหญ่ ราคา 12.00 บาท</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/70Hbg7eYsX</t>
+          <t>https://s.shopee.co.th/7KuS4ggUuo</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98w-lyel2mw8dhfla5.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-81zuh-mn13pkf6h0qte8.webp</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -1711,46 +1705,46 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>104</v>
+        <v>1</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>🔥(120*70CM) แผ่นดักทรายแมว พรมดักทรายแมว พรม 2 ชั้น EVA ช่วยดัก ทรายแมว ที่ติดตามเท้า แผ่น รอง ทรายแมว ขนาด ใหญ่ ราคา 12.00 บาท</t>
+          <t>F&amp;G วิลล่าแมว Cat Villa บ้านแมว กรงแมว วิลล่าไม้เนื้อแข็งตู้แมว ตู้โชว์ไม้เนื้อแข็ง วิลล่าแมวขนาดใหญ จัดส่งภายใน24ชั่วโม ราคา 1999.00 บาท</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7KuS4ggUuo</t>
+          <t>https://s.shopee.co.th/20svidIbiq</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-81zuh-mn13pkf6h0qte8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m3ytl0pibu8a95.webp</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>done 2026-06-15 05:50</t>
+          <t>done 2026-06-15 05:51</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1</v>
+        <v>120</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>F&amp;G วิลล่าแมว Cat Villa บ้านแมว กรงแมว วิลล่าไม้เนื้อแข็งตู้แมว ตู้โชว์ไม้เนื้อแข็ง วิลล่าแมวขนาดใหญ จัดส่งภายใน24ชั่วโม ราคา 1999.00 บาท</t>
+          <t>ถุงเก็บมูลสัตว์เลี้ยง อึหมา แมว ถุงขยะ ถุงเก็บอึหมา♻ย่อยสลายได้เองโดยธรรมชาติ ถุงเก็บอึแมว/สุนัขและสัตว์เลี้ยง ราคา 39.00 บาท</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/20svidIbiq</t>
+          <t>https://s.shopee.co.th/3B4t746pHm</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m3ytl0pibu8a95.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0p-mb535hvzw3sm83.webp</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -1761,21 +1755,21 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>120</v>
+        <v>72</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ถุงเก็บมูลสัตว์เลี้ยง อึหมา แมว ถุงขยะ ถุงเก็บอึหมา♻ย่อยสลายได้เองโดยธรรมชาติ ถุงเก็บอึแมว/สุนัขและสัตว์เลี้ยง ราคา 39.00 บาท</t>
+          <t>Gager (10 กิโล) ทรายแมวภูเขาไฟ ทรายแมวเบนโทไนท์ Bentonite ดับกลิ่นได้ดีเยี่ยม เกรดพรีเมียม ราคา 489.00 บาท</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3B4t746pHm</t>
+          <t>https://s.shopee.co.th/80A8rpVK8s</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0p-mb535hvzw3sm83.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-23020-m46dux2nqsnv37.webp</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -1786,71 +1780,71 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Gager (10 กิโล) ทรายแมวภูเขาไฟ ทรายแมวเบนโทไนท์ Bentonite ดับกลิ่นได้ดีเยี่ยม เกรดพรีเมียม ราคา 489.00 บาท</t>
+          <t>yoyopet : น้ำยาเช็ดหู ที่หยอดหูแมว ทำความสะอาดหู ปลอดภัย ใช้ได้ทั้งหมาและแมว มี 2 ขนาด 60 / 120 ml ราคา 60.00 บาท</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/80A8rpVK8s</t>
+          <t>https://s.shopee.co.th/2qS2iPnWVW</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-23020-m46dux2nqsnv37.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0q-mbf3w9n5hoyj3a.webp</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>done 2026-06-15 05:51</t>
+          <t>done 2026-06-16 06:24</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>103</v>
+        <v>16</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>yoyopet : น้ำยาเช็ดหู ที่หยอดหูแมว ทำความสะอาดหู ปลอดภัย ใช้ได้ทั้งหมาและแมว มี 2 ขนาด 60 / 120 ml ราคา 60.00 บาท</t>
+          <t>คอกกระบะฮันเตอร์(Hunter Cage) ราคา 11715.00 บาท</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qS2iPnWVW</t>
+          <t>https://s.shopee.co.th/gNUc3Zcns</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0q-mbf3w9n5hoyj3a.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul0-lfgefx1hi2su42.webp</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>done 2026-06-16 06:24</t>
+          <t>done 2026-06-16 06:25</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>16</v>
+        <v>83</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>คอกกระบะฮันเตอร์(Hunter Cage) ราคา 11715.00 บาท</t>
+          <t>สเปรย์น้ำหอมระงับกลิ่น แบรนด์พราวพาว สูตรอ่อนโยน สารสกัดจากธรรมชาติ 3 กลิ่น หอมละมุนชื่นใจ ราคา 169.00 บาท</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/gNUc3Zcns</t>
+          <t>https://s.shopee.co.th/5VSntGZdL7</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul0-lfgefx1hi2su42.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m2usz5kign3644.webp</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -1861,21 +1855,21 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>สเปรย์น้ำหอมระงับกลิ่น แบรนด์พราวพาว สูตรอ่อนโยน สารสกัดจากธรรมชาติ 3 กลิ่น หอมละมุนชื่นใจ ราคา 169.00 บาท</t>
+          <t>F&amp;G คอนโดแมว cat tree คอนโดไม้ ไม้แท้ ที่นอนแมว ไม่ใช้พื้นที่ มั่นคงไม่สั่นคลอน ของเล่นแมว ราคา 2132.00 บาท</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5VSntGZdL7</t>
+          <t>https://s.shopee.co.th/7VDsGxBScD</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m2usz5kign3644.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-monqurfriknfb7.webp</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -1886,21 +1880,21 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>F&amp;G คอนโดแมว cat tree คอนโดไม้ ไม้แท้ ที่นอนแมว ไม่ใช้พื้นที่ มั่นคงไม่สั่นคลอน ของเล่นแมว ราคา 2132.00 บาท</t>
+          <t>me-o delite มีโอดีไลท์ อาหารเปียกแมว มีโอดีไลท์ 70g.x12ซอง (1โหล)สินค้าพร้อมจัดส่ง ราคา 280.00 บาท</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7VDsGxBScD</t>
+          <t>https://s.shopee.co.th/4qD7665l3G</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-monqurfriknfb7.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/b6f6b78245b02c906da9bcc8db6d65c5.webp</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -1911,46 +1905,46 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>me-o delite มีโอดีไลท์ อาหารเปียกแมว มีโอดีไลท์ 70g.x12ซอง (1โหล)สินค้าพร้อมจัดส่ง ราคา 280.00 บาท</t>
+          <t>ความจุขนาดใหญ่พิเศษ กะบะทรายแมว ห้องน้ำแมวใหญ่ ห้องน้ำแมว กระบะทรายแมว ของใช้แมว รุ่นขอบสูงมีตะแกรงดักทราย ราคา 87.00 บาท</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4qD7665l3G</t>
+          <t>https://s.shopee.co.th/3qKZuGRiIG</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/b6f6b78245b02c906da9bcc8db6d65c5.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mjf9apq6hm2qa6.webp</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>done 2026-06-16 06:25</t>
+          <t>done 2026-06-17 06:10</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>108</v>
+        <v>13</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ความจุขนาดใหญ่พิเศษ กะบะทรายแมว ห้องน้ำแมวใหญ่ ห้องน้ำแมว กระบะทรายแมว ของใช้แมว รุ่นขอบสูงมีตะแกรงดักทราย ราคา 87.00 บาท</t>
+          <t>PANDO Second Generation Pet Trolleyแพนโด้ รถเข็นสำหรับสัตว์เลี้ยง เวอร์ชันอัพเกรด ราคา 3390.00 บาท</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qKZuGRiIG</t>
+          <t>https://s.shopee.co.th/110OWov8hV</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mjf9apq6hm2qa6.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mp208h070r2883.webp</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -1961,21 +1955,21 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PANDO Second Generation Pet Trolleyแพนโด้ รถเข็นสำหรับสัตว์เลี้ยง เวอร์ชันอัพเกรด ราคา 3390.00 บาท</t>
+          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology เครื่องให้อาหารอัตโนมัติ เก็บสถิติการกิน ควบคุมผ่านแอป CATLINK Fresh 2 ราคา 5992.00 บาท</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/110OWov8hV</t>
+          <t>https://s.shopee.co.th/LkhjcTaFu</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mp208h070r2883.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0t-mbdq486x43gh65.webp</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -1986,21 +1980,21 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>21</v>
+        <v>121</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology เครื่องให้อาหารอัตโนมัติ เก็บสถิติการกิน ควบคุมผ่านแอป CATLINK Fresh 2 ราคา 5992.00 บาท</t>
+          <t>😻ที่ลับเล็บแมว คอนโดแมว💒 บ้านแมว ลับเล็บแมว กล่องแมว เตียงแมวสามารถรองรับแมวได้ 3-4 ตัว คอนโดแมว บ้านลับเล็บแมว กล่องแมว ราคา 166.00 บาท</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/LkhjcTaFu</t>
+          <t>https://s.shopee.co.th/2VpCJqjSJ0</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0t-mbdq486x43gh65.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-ma12cstnwlsfed.webp</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2011,21 +2005,21 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>😻ที่ลับเล็บแมว คอนโดแมว💒 บ้านแมว ลับเล็บแมว กล่องแมว เตียงแมวสามารถรองรับแมวได้ 3-4 ตัว คอนโดแมว บ้านลับเล็บแมว กล่องแมว ราคา 166.00 บาท</t>
+          <t>ดีย์ ฟล็อคซ์ อาหารกบ 20kg.** ( 3762 / 3763 / 3764 ) ราคา 770.00 บาท</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2VpCJqjSJ0</t>
+          <t>https://s.shopee.co.th/5fmE5az3ux</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-ma12cstnwlsfed.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/3fe3471908638668e5d1ea1240c36a51.webp</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2036,46 +2030,46 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>94</v>
+        <v>20</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ดีย์ ฟล็อคซ์ อาหารกบ 20kg.** ( 3762 / 3763 / 3764 ) ราคา 770.00 บาท</t>
+          <t>Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK Lite ราคา 8800.00 บาท</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5fmE5az3ux</t>
+          <t>https://s.shopee.co.th/9zvDFNIgyY</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/3fe3471908638668e5d1ea1240c36a51.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-mauvmoz6b0omd5.webp</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>done 2026-06-17 06:10</t>
+          <t>done 2026-06-19 06:24</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK Lite ราคา 8800.00 บาท</t>
+          <t>PANDO Second Generation Cat Litter Box (Lite) ห้องน้ำแมวอัตโนมัติรุ่น 2 ราคา 8990.00 บาท</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9zvDFNIgyY</t>
+          <t>https://s.shopee.co.th/2BCLv5rnUp</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-mauvmoz6b0omd5.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mp2024pophcc13.webp</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2086,21 +2080,21 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PANDO Second Generation Cat Litter Box (Lite) ห้องน้ำแมวอัตโนมัติรุ่น 2 ราคา 8990.00 บาท</t>
+          <t>มีโอ โกลด์ อาหารแมว แมวเลี้ยงในบ้าน (1.2 กิโลกรัม) | Me-O Gold Indoor Cat (1.2 kg.) ราคา 229.00 บาท</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2BCLv5rnUp</t>
+          <t>https://s.shopee.co.th/5ApxUdXjQO</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mp2024pophcc13.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/d8dbbb26ca1090acfb78f8339cf37106.webp</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2111,46 +2105,46 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>78</v>
+        <v>125</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>มีโอ โกลด์ อาหารแมว แมวเลี้ยงในบ้าน (1.2 กิโลกรัม) | Me-O Gold Indoor Cat (1.2 kg.) ราคา 229.00 บาท</t>
+          <t>jaywa กระเป๋าแมวล้อลากสะพายเป้ ใส่แมวตัวใหญ่ หมาเล็ก แมวเมนคูน ขึ้นบันไดเลื่อน เข้าลิฟท์ อยู่คอนโด ราคา 2372.00 บาท</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5ApxUdXjQO</t>
+          <t>https://s.shopee.co.th/4AxQIv75Fv</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/d8dbbb26ca1090acfb78f8339cf37106.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m9q3mvzvdka9df.webp</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>done 2026-06-19 06:24</t>
+          <t>done 2026-06-19 06:25</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>jaywa กระเป๋าแมวล้อลากสะพายเป้ ใส่แมวตัวใหญ่ หมาเล็ก แมวเมนคูน ขึ้นบันไดเลื่อน เข้าลิฟท์ อยู่คอนโด ราคา 2372.00 บาท</t>
+          <t>(12ซอง)Lola&amp;Co โลล่าแอนด์โค อาหารเปียกแมว สูตร Complete &amp; Balanced เกรนฟรี ไม่เติมเกลือ ขนาด 80g. 12ซอง ราคา 210.00 บาท</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4AxQIv75Fv</t>
+          <t>https://s.shopee.co.th/W47vt8AfV</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m9q3mvzvdka9df.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98r-lp5dhkayuida56.webp</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2161,46 +2155,46 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>(12ซอง)Lola&amp;Co โลล่าแอนด์โค อาหารเปียกแมว สูตร Complete &amp; Balanced เกรนฟรี ไม่เติมเกลือ ขนาด 80g. 12ซอง ราคา 210.00 บาท</t>
+          <t>yoyopet : แผ่นเช็ดคราบน้ำตาสุนัขและแมว บรรจุ130แผ่น Pet wipes ทิชชู่เปียกเช็ดคราบน้ำตา ราคา 52.00 บาท</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/W47vt8AfV</t>
+          <t>https://s.shopee.co.th/50WXIIYtnz</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98r-lp5dhkayuida56.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m30f4f0ikpqkea.webp</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>done 2026-06-19 06:25</t>
+          <t>done 2026-06-19 07:40</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>yoyopet : แผ่นเช็ดคราบน้ำตาสุนัขและแมว บรรจุ130แผ่น Pet wipes ทิชชู่เปียกเช็ดคราบน้ำตา ราคา 52.00 บาท</t>
+          <t>DIGITAL PET Automatic cat litter box ห้องน้ำแมวอัตโนมัติOpen-top และแอปควบคุมระยะไกล WithCamera ห้องน้ำเเมวแบบอัตโนมัติ ราคา 4299.00 บาท</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/50WXIIYtnz</t>
+          <t>https://s.shopee.co.th/3B4t6rlLOH</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m30f4f0ikpqkea.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zti-mes9b8c97mrq22.webp</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2211,21 +2205,21 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>40</v>
+        <v>101</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>DIGITAL PET Automatic cat litter box ห้องน้ำแมวอัตโนมัติOpen-top และแอปควบคุมระยะไกล WithCamera ห้องน้ำเเมวแบบอัตโนมัติ ราคา 4299.00 บาท</t>
+          <t>คอกกระบะฮันเตอร์(Hunter Cage) ราคา 12089.00 บาท</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3B4t6rlLOH</t>
+          <t>https://s.shopee.co.th/2BCLvBXqMM</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zti-mes9b8c97mrq22.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul0-lfgefx1hi2su42.webp</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2236,21 +2230,21 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>คอกกระบะฮันเตอร์(Hunter Cage) ราคา 12089.00 บาท</t>
+          <t>คอกสัตว์เลี้ยง กรงสัตว์เลี้ยง พับได้ พื้นที่ขนาดใหญ่ ห้องคลอดแมวสี่เหลี่ยมปิด คอกแมว คอกสุนัข ราคา 409.00 บาท</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2BCLvBXqMM</t>
+          <t>https://s.shopee.co.th/6VLL56G5GE</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul0-lfgefx1hi2su42.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/cn-11134207-7r98o-lv4jadivnf6c2b.webp</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2261,21 +2255,21 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>คอกสัตว์เลี้ยง กรงสัตว์เลี้ยง พับได้ พื้นที่ขนาดใหญ่ ห้องคลอดแมวสี่เหลี่ยมปิด คอกแมว คอกสุนัข ราคา 409.00 บาท</t>
+          <t>PIDAN Pet Bed Alumi Grey กระทะเย็นอะลูมิเนียม ที่นอนแมวเย็น กะทะแมวเย็น ราคา 1900.00 บาท</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6VLL56G5GE</t>
+          <t>https://s.shopee.co.th/6pyBTfBcwv</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/cn-11134207-7r98o-lv4jadivnf6c2b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134201-7r98v-lyah4te3ab2900.webp</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2286,46 +2280,46 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PIDAN Pet Bed Alumi Grey กระทะเย็นอะลูมิเนียม ที่นอนแมวเย็น กะทะแมวเย็น ราคา 1900.00 บาท</t>
+          <t>[ส่งฟรี+แถม2กป] ChooChoo ชูชู สมูทตี้ปลาแซลมอน สูตรบำรุงเลือด 24 กระป๋อง (80กรัมx24กระป๋อง) ราคา 862.00 บาท</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6pyBTfBcwv</t>
+          <t>https://s.shopee.co.th/2qS2iKda5q</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134201-7r98v-lyah4te3ab2900.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r992-luancixsfmkx2d.webp</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>done 2026-06-19 07:40</t>
+          <t>done 2026-06-20 05:38</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>70</v>
+        <v>124</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>[ส่งฟรี+แถม2กป] ChooChoo ชูชู สมูทตี้ปลาแซลมอน สูตรบำรุงเลือด 24 กระป๋อง (80กรัมx24กระป๋อง) ราคา 862.00 บาท</t>
+          <t>ทรายแมว ครอกแมวเบนโทไนท์ มี 6 กลิ่นให้เลือก พลังฆ่ากลิ่นที่เหนือกว่า การดูดซับที่แข็งแกร่ง 6L/2KG ราคา 38.00 บาท</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qS2iKda5q</t>
+          <t>https://s.shopee.co.th/9fIMr1dPnc</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r992-luancixsfmkx2d.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lzub9j05k9ex02.webp</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2336,21 +2330,21 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>124</v>
+        <v>43</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ทรายแมว ครอกแมวเบนโทไนท์ มี 6 กลิ่นให้เลือก พลังฆ่ากลิ่นที่เหนือกว่า การดูดซับที่แข็งแกร่ง 6L/2KG ราคา 38.00 บาท</t>
+          <t>[Doctor By CAT BREATH] อาหารเสริมลมหายใจสัตว์เลี้ยงแมว Churu อาหารเปียกรักษา (30 แท่ง) ราคา 1513.00 บาท</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fIMr1dPnc</t>
+          <t>https://s.shopee.co.th/8KmzGNJ9uv</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lzub9j05k9ex02.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134207-81ztz-mmu2tg1y3tvq52.webp</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2361,21 +2355,21 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>[Doctor By CAT BREATH] อาหารเสริมลมหายใจสัตว์เลี้ยงแมว Churu อาหารเปียกรักษา (30 แท่ง) ราคา 1513.00 บาท</t>
+          <t>คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุนัขและแมว สูตร Fit&amp;Firm ฟิต&amp;เฟิร์มบำรุงหัวใจ ราคา 490.00 บาท</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8KmzGNJ9uv</t>
+          <t>https://s.shopee.co.th/4ftgtbShWq</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134207-81ztz-mmu2tg1y3tvq52.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lxa2x1xet5n38c.webp</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2386,21 +2380,21 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>31</v>
+        <v>130</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุนัขและแมว สูตร Fit&amp;Firm ฟิต&amp;เฟิร์มบำรุงหัวใจ ราคา 490.00 บาท</t>
+          <t>[ส่งฟรี+แถม2กป] ชูชูสมูทตี้ อาหารบำรุงแมว สูตรไข่ขาวดูแลไต24กระป๋อง ทานง่าย หอม อร่อย ราคา 862.00 บาท</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4ftgtbShWq</t>
+          <t>https://s.shopee.co.th/7fXITMXYyu</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lxa2x1xet5n38c.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98w-luanf4e1og0hfc.webp</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2411,46 +2405,46 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>130</v>
+        <v>102</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>[ส่งฟรี+แถม2กป] ชูชูสมูทตี้ อาหารบำรุงแมว สูตรไข่ขาวดูแลไต24กระป๋อง ทานง่าย หอม อร่อย ราคา 862.00 บาท</t>
+          <t>Pawdy อาหารสุนัขเกรดพรีเมียม Holistic สำหรับสุนัขโต อายุ 1-6 ปี สูตรเนื้อวัวย่างและเห็ดทรัฟเฟิล ขนาด 8 กก. (มี 2 ขนาด) ราคา 1278.00 บาท</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7fXITMXYyu</t>
+          <t>https://s.shopee.co.th/8ATZ4DLj5r</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98w-luanf4e1og0hfc.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mn6zvfws7coy54.webp</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>done 2026-06-20 05:38</t>
+          <t>done 2026-06-21 05:49</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>102</v>
+        <v>56</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Pawdy อาหารสุนัขเกรดพรีเมียม Holistic สำหรับสุนัขโต อายุ 1-6 ปี สูตรเนื้อวัวย่างและเห็ดทรัฟเฟิล ขนาด 8 กก. (มี 2 ขนาด) ราคา 1278.00 บาท</t>
+          <t>Petcho แผ่นรองฉี่ แผ่นรองฉี่สุนัข แผ่นรองฉี่สัตว์เลี้ยง ที่ซับฉี่ สุนัข แมว ซุปเปอร์ดูดซับ 7 ชั้นแ ลายน่ารัก Pet Pad ราคา 177.00 บาท</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8ATZ4DLj5r</t>
+          <t>https://s.shopee.co.th/4qD75yE4nh</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mn6zvfws7coy54.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasg-m51cigt961iibd.webp</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -2461,46 +2455,46 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>56</v>
+        <v>129</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Petcho แผ่นรองฉี่ แผ่นรองฉี่สุนัข แผ่นรองฉี่สัตว์เลี้ยง ที่ซับฉี่ สุนัข แมว ซุปเปอร์ดูดซับ 7 ชั้นแ ลายน่ารัก Pet Pad ราคา 177.00 บาท</t>
+          <t>กรง สแตนเลส 304 กรงสัตว์เลี้ยงขนาดใหญ่（125*110cm）กรงสแตนเลส กรงสุนัขพับได้ กรงสุนัข คอกกรงสัตว์เลี้ยง dog cages crates ราคา 2667.00 บาท</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4qD75yE4nh</t>
+          <t>https://s.shopee.co.th/qgyKnqQa2</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasg-m51cigt961iibd.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r992-lya8q6n2fnah9e.webp</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>done 2026-06-21 05:49</t>
+          <t>done 2026-06-21 05:50</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>129</v>
+        <v>7</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>กรง สแตนเลส 304 กรงสัตว์เลี้ยงขนาดใหญ่（125*110cm）กรงสแตนเลส กรงสุนัขพับได้ กรงสุนัข คอกกรงสัตว์เลี้ยง dog cages crates ราคา 2667.00 บาท</t>
+          <t>NaviPet Grooming Vacuum KIT 7 in 1 เครื่องปัตตาเลียนตัดแต่งขนสำหรับสัตว์เลี้ยง และดูดฝุ่น กรูมมิ่งสำหรับดูด ราคา 2590.00 บาท</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/qgyKnqQa2</t>
+          <t>https://s.shopee.co.th/40e06K2cCJ</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r992-lya8q6n2fnah9e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasc-madx77cb5x8wff.webp</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -2511,21 +2505,21 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>NaviPet Grooming Vacuum KIT 7 in 1 เครื่องปัตตาเลียนตัดแต่งขนสำหรับสัตว์เลี้ยง และดูดฝุ่น กรูมมิ่งสำหรับดูด ราคา 2590.00 บาท</t>
+          <t>Petology คอนโดแมวคุณภาพสูง แข็งแรง ทนทาน ใช้งานได้นาน รุ่น CD-01 ราคา 11000.00 บาท</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/40e06K2cCJ</t>
+          <t>https://s.shopee.co.th/1qZVWPYkhV</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasc-madx77cb5x8wff.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0i-mbdqw6sm2nna5d.webp</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -2536,46 +2530,46 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>37</v>
+        <v>119</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Petology คอนโดแมวคุณภาพสูง แข็งแรง ทนทาน ใช้งานได้นาน รุ่น CD-01 ราคา 11000.00 บาท</t>
+          <t>【BUFFO】ผ้าเช็ดทำความสะอาดสัตว์เลี้ยง 80 แผ่น สุนัขและแมว ปลอดภัย สำหรับเช็ดสัต ว์เลี้ยง ทิชชู่เปียก กำจัดกลิ่นแบคทีเรีย ราคา 12.00 บาท</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1qZVWPYkhV</t>
+          <t>https://s.shopee.co.th/9fIMr0eIfj</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0i-mbdqw6sm2nna5d.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98y-lnsaey0d1p47d4.webp</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>done 2026-06-21 05:50</t>
+          <t>done 2026-06-22 05:49</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>119</v>
+        <v>1</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>【BUFFO】ผ้าเช็ดทำความสะอาดสัตว์เลี้ยง 80 แผ่น สุนัขและแมว ปลอดภัย สำหรับเช็ดสัต ว์เลี้ยง ทิชชู่เปียก กำจัดกลิ่นแบคทีเรีย ราคา 12.00 บาท</t>
+          <t>ยกโหล Nekko อาหารเปียกแมว 70 กรัม12ซอง ราคา 158.00 บาท</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fIMr0eIfj</t>
+          <t>https://s.shopee.co.th/7AayLy4TAu</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98y-lnsaey0d1p47d4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823r0-mp0pjfpweby84e.webp</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -2586,21 +2580,21 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ยกโหล Nekko อาหารเปียกแมว 70 กรัม12ซอง ราคา 158.00 บาท</t>
+          <t>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI ราคา 7714.00 บาท</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7AayLy4TAu</t>
+          <t>https://s.shopee.co.th/4VaGhEZh87</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823r0-mp0pjfpweby84e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -2611,21 +2605,21 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>4</v>
+        <v>54</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI ราคา 7714.00 บาท</t>
+          <t>[ส่งฟรี+แถม2กป] ชูชู อาหารเสริมแมวสมูทตี้สูตรปลาคัตสึโอะ 24กระป๋อง บำรุงเข้มข้น ด้วยไฮโดรไลซ์โปรตีนจากประเทศเบลเยี่ยม ราคา 862.00 บาท</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4VaGhEZh87</t>
+          <t>https://s.shopee.co.th/60P4U6vgCO</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98v-luan6o2wzyddfc.webp</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -2636,21 +2630,21 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>54</v>
+        <v>118</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>[ส่งฟรี+แถม2กป] ชูชู อาหารเสริมแมวสมูทตี้สูตรปลาคัตสึโอะ 24กระป๋อง บำรุงเข้มข้น ด้วยไฮโดรไลซ์โปรตีนจากประเทศเบลเยี่ยม ราคา 862.00 บาท</t>
+          <t>[ขายดี] สมาร์ทฮาร์ท อาหารสุนัข สุนัขโต รสเนื้ออบ 10 กก. / SmartHeart Adult Roast Beef 10kg ราคา 819.00 บาท</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/60P4U6vgCO</t>
+          <t>https://s.shopee.co.th/70Hbg6gXva</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98v-luan6o2wzyddfc.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m682zid86p6f5f.webp</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -2661,46 +2655,46 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>118</v>
+        <v>73</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>[ขายดี] สมาร์ทฮาร์ท อาหารสุนัข สุนัขโต รสเนื้ออบ 10 กก. / SmartHeart Adult Roast Beef 10kg ราคา 819.00 บาท</t>
+          <t>NAVIPET Wireless Drinking Fountain V1 น้ำพุไร้สายความจุ2.5ลิตร มีแบตในตัว5000 mAh ประกันศูนย์ไทย1 ปี ราคา 742.00 บาท</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/70Hbg6gXva</t>
+          <t>https://s.shopee.co.th/gNY8M5yK7</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m682zid86p6f5f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mf998jaiwff3bb.webp</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>done 2026-06-22 05:49</t>
+          <t>done 2026-06-23 06:06</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>NAVIPET Wireless Drinking Fountain V1 น้ำพุไร้สายความจุ2.5ลิตร มีแบตในตัว5000 mAh ประกันศูนย์ไทย1 ปี ราคา 742.00 บาท</t>
+          <t>วิลล่าแมวไม้ บ้านแมว กรงสัตว์เลี้ยง อพาร์ตเมนท์แมวไม้ อพาร์ตเมนท์แมวไม้เนื้อแข็ง กรงสัตว์เลี้ยง วิลล่าแมวไม้ ราคา 1329.00 บาท</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/gNY8M5yK7</t>
+          <t>https://s.shopee.co.th/40e06XRXji</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mf998jaiwff3bb.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasl-m1e5ujd17j5bac.webp</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -2711,21 +2705,21 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>97</v>
+        <v>15</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>วิลล่าแมวไม้ บ้านแมว กรงสัตว์เลี้ยง อพาร์ตเมนท์แมวไม้ อพาร์ตเมนท์แมวไม้เนื้อแข็ง กรงสัตว์เลี้ยง วิลล่าแมวไม้ ราคา 1329.00 บาท</t>
+          <t>แมว ไดร์เป่าผม 62 /82L ของใช้แมว เครื่องเป่าขนแมว อาบน้ําแมว ตู้อบแมว ตั้งเวลาได้ ไดร์เป่าขนแมว ราคา 2933.00 บาท</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/40e06XRXji</t>
+          <t>https://s.shopee.co.th/9fIJKasq1a</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasl-m1e5ujd17j5bac.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134201-7rasf-maxkg8lg2suo1b.webp</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -2736,21 +2730,21 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>แมว ไดร์เป่าผม 62 /82L ของใช้แมว เครื่องเป่าขนแมว อาบน้ําแมว ตู้อบแมว ตั้งเวลาได้ ไดร์เป่าขนแมว ราคา 2933.00 บาท</t>
+          <t>Petlover ธัญพืชผสมพิเศษกว่า 35+ ชนิด สำหรับนกวัยหัดแทะ และนกแก้วทุกสายพันธุ์ (แบ่งขาย 500G / 1KG) ราคา 24.00 บาท</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fIJKasq1a</t>
+          <t>https://s.shopee.co.th/20svidVjns</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134201-7rasf-maxkg8lg2suo1b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mn2op1vp4d1dba.webp</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -2761,21 +2755,21 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>2</v>
+        <v>71</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Petlover ธัญพืชผสมพิเศษกว่า 35+ ชนิด สำหรับนกวัยหัดแทะ และนกแก้วทุกสายพันธุ์ (แบ่งขาย 500G / 1KG) ราคา 24.00 บาท</t>
+          <t>เสื้อน้องหมาลาย เครื่องปรุงรส ผ้าไมโครสีสันสดใสพร้อมส่ง ราคา 50.00 บาท</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/20svidVjns</t>
+          <t>https://s.shopee.co.th/6pyBTgRAjL</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mn2op1vp4d1dba.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m96tiq9mlglrc3.webp</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -2786,46 +2780,46 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>เสื้อน้องหมาลาย เครื่องปรุงรส ผ้าไมโครสีสันสดใสพร้อมส่ง ราคา 50.00 บาท</t>
+          <t>[ ตกกิโลละ 119 บาท l ไซส์กระสอบ 15 กิโล ] petheria อาหารสุนัขแบบเม็ดเกรด SUPER PREMIUM มีให้เลือกทุกช่วงวัย ราคา 1798.00 บาท</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6pyBTgRAjL</t>
+          <t>https://s.shopee.co.th/70HbfvolrB</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m96tiq9mlglrc3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98w-lwv3eh1w2dan86.webp</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>done 2026-06-23 06:06</t>
+          <t>done 2026-06-24 05:51</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>[ ตกกิโลละ 119 บาท l ไซส์กระสอบ 15 กิโล ] petheria อาหารสุนัขแบบเม็ดเกรด SUPER PREMIUM มีให้เลือกทุกช่วงวัย ราคา 1798.00 บาท</t>
+          <t>JOOM ' S SHAMPOO แชมพูสำหรับสุนัขและแมว ขนาด 250ml. สูตรอ่อนโยน ไม่มีสารอันตราย ราคา 259.00 บาท</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/70HbfvolrB</t>
+          <t>https://s.shopee.co.th/5fmE5Vc3go</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98w-lwv3eh1w2dan86.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0t-mbewxjfiaqo113.webp</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -2836,21 +2830,21 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>JOOM ' S SHAMPOO แชมพูสำหรับสุนัขและแมว ขนาด 250ml. สูตรอ่อนโยน ไม่มีสารอันตราย ราคา 259.00 บาท</t>
+          <t>yoyopet : ถุงมือสปา อาบน้ำแมว สุนัข ทำความสะอาดสัตว์เลี้ยง ใช้งานง่าย กลิ่นหอม ไม่ระคายเคืองผิว ราคา 60.00 บาท</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5fmE5Vc3go</t>
+          <t>https://s.shopee.co.th/2BCLvDXvgD</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0t-mbewxjfiaqo113.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasf-m89uuwmiz8sv02.webp</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -2861,46 +2855,46 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>115</v>
+        <v>67</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>yoyopet : ถุงมือสปา อาบน้ำแมว สุนัข ทำความสะอาดสัตว์เลี้ยง ใช้งานง่าย กลิ่นหอม ไม่ระคายเคืองผิว ราคา 60.00 บาท</t>
+          <t>yoyopet : Furry Fresh สเปรย์ปรับอากาศ สเปรย์น้ำหอม ดับกลิ่นฉี่แมวและสัตว์เลี้ยง ปลอดภัย 500ml ราคา 86.00 บาท</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2BCLvDXvgD</t>
+          <t>https://s.shopee.co.th/9fIMqslrYK</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasf-m89uuwmiz8sv02.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mlsx7eyhi61190.webp</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>done 2026-06-24 05:51</t>
+          <t>done 2026-06-24 05:52</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>yoyopet : Furry Fresh สเปรย์ปรับอากาศ สเปรย์น้ำหอม ดับกลิ่นฉี่แมวและสัตว์เลี้ยง ปลอดภัย 500ml ราคา 86.00 บาท</t>
+          <t>Pet Record ผ้าเช็ดทำความสะอาดสัตว์เลี้ยง 80 แผ่น สุนัขและแมว ปลอดภัย สำหรับเช็ดสัต ว์เลี้ยง ราคา 11.00 บาท</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fIMqslrYK</t>
+          <t>https://s.shopee.co.th/3g19hu8nZv</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mlsx7eyhi61190.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mlx518xkyght72.webp</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -2911,46 +2905,46 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>87</v>
+        <v>8</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Pet Record ผ้าเช็ดทำความสะอาดสัตว์เลี้ยง 80 แผ่น สุนัขและแมว ปลอดภัย สำหรับเช็ดสัต ว์เลี้ยง ราคา 11.00 บาท</t>
+          <t>Petology คอนโดแมวคุณภาพสูง แข็งแรง ทนทาน ใช้งานได้นาน รุ่น CD-01 ราคา 11000.00 บาท</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3g19hu8nZv</t>
+          <t>https://s.shopee.co.th/40dwaAECCx</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mlx518xkyght72.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0i-mbdqw6sm2nna5d.webp</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>done 2026-06-24 05:52</t>
+          <t>done 2026-06-25 05:52</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>8</v>
+        <v>74</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Petology คอนโดแมวคุณภาพสูง แข็งแรง ทนทาน ใช้งานได้นาน รุ่น CD-01 ราคา 11000.00 บาท</t>
+          <t>Pawdy อาหารสุนัขเกรดพรีเมียม สำหรับสุนัขสูงวัย อายุมากกว่า 7 ปี สูตรแกะและปลา ผสมเนื้อจระเข้ ขนาด 1.2 กก. ราคา 333.00 บาท</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/40dwaAECCx</t>
+          <t>https://s.shopee.co.th/4LGqV615Un</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0i-mbdqw6sm2nna5d.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mn9tb9drwvszd2.webp</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -2961,21 +2955,21 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Pawdy อาหารสุนัขเกรดพรีเมียม สำหรับสุนัขสูงวัย อายุมากกว่า 7 ปี สูตรแกะและปลา ผสมเนื้อจระเข้ ขนาด 1.2 กก. ราคา 333.00 บาท</t>
+          <t>My Paws น้ำยาล้างจาน น้ำยาล้างของเล่น น้ำยาล้างจานสำหรับสัตว์เลี้ยง สารสกัดจากธรรมชาติ อ่อนโยน สำหรับสัตว์เลี้ยงทุกชนิด ราคา 38.00 บาท</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4LGqV615Un</t>
+          <t>https://s.shopee.co.th/1Vwf7wPVkj</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mn9tb9drwvszd2.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mp37aagvwj5te3.webp</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -2986,46 +2980,46 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>My Paws น้ำยาล้างจาน น้ำยาล้างของเล่น น้ำยาล้างจานสำหรับสัตว์เลี้ยง สารสกัดจากธรรมชาติ อ่อนโยน สำหรับสัตว์เลี้ยงทุกชนิด ราคา 38.00 บาท</t>
+          <t>Dog Days อาหารสุนัขรสปลา (2.8 kg) Derma เกรด Holistic สูตรสำหรับแพ้ไก่โดยเฉพาะ โซเดียมต่ำ ราคา 521.00 บาท</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1Vwf7wPVkj</t>
+          <t>https://s.shopee.co.th/gNY8Pn242</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mp37aagvwj5te3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-modf6uepclcd05.webp</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>done 2026-06-25 05:52</t>
+          <t>done 2026-06-25 05:53</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Dog Days อาหารสุนัขรสปลา (2.8 kg) Derma เกรด Holistic สูตรสำหรับแพ้ไก่โดยเฉพาะ โซเดียมต่ำ ราคา 521.00 บาท</t>
+          <t>หวีขนแมว แปรงขนแมว หวีแมว แปรงขนสุนัข แปลงขนแมว หวีขนสุนัข ที่หวีขนแมว กําจัดขนแมว มีปุ่มดันขนออก ราคา 25.00 บาท</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/gNY8Pn242</t>
+          <t>https://s.shopee.co.th/20svirqkvK</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-modf6uepclcd05.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134211-7rasi-maurrwfy4mt0ec.webp</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -3036,71 +3030,71 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>99</v>
+        <v>68</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>หวีขนแมว แปรงขนแมว หวีแมว แปรงขนสุนัข แปลงขนแมว หวีขนสุนัข ที่หวีขนแมว กําจัดขนแมว มีปุ่มดันขนออก ราคา 25.00 บาท</t>
+          <t>Petcho แผ่นรองฉี่ แผ่นรองฉี่สุนัข แผ่นรองซับ สัตว์เลี้ยง ซับได้มาก พลังการดูดซับ 6ชั้น ช่วยฝึกขับถ่าย ราคา 149.00 บาท</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/20svirqkvK</t>
+          <t>https://s.shopee.co.th/W47w2T99w</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134211-7rasi-maurrwfy4mt0ec.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98t-lyelrzpqov41c6.webp</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>done 2026-06-25 05:53</t>
+          <t>done 2026-06-26 06:02</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Petcho แผ่นรองฉี่ แผ่นรองฉี่สุนัข แผ่นรองซับ สัตว์เลี้ยง ซับได้มาก พลังการดูดซับ 6ชั้น ช่วยฝึกขับถ่าย ราคา 149.00 บาท</t>
+          <t>[VetPlus] SAMYLIN Small Breed for Dogs &amp; Cats (30 Tablets/Sachets) / Nutritional Supplement for Healthy Liver Function ราคา 2184.00 บาท</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/W47w2T99w</t>
+          <t>https://s.shopee.co.th/9zvDFSl7uu</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98t-lyelrzpqov41c6.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134207-7rd5l-m70gtvlk15ck4a.webp</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>done 2026-06-26 06:02</t>
+          <t>done 2026-06-26 06:03</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>[VetPlus] SAMYLIN Small Breed for Dogs &amp; Cats (30 Tablets/Sachets) / Nutritional Supplement for Healthy Liver Function ราคา 2184.00 บาท</t>
+          <t>BIO น้ำยาดับกลิ่น กลิ่นฉี่ กลิ่นมูลสัตว์เลี้ยง ล้างพื้นกลิ่นฉี่ ทำความสะอาด ปราศจากเชื้อโรค กลิ่นโอโซนบริสุทธิ์ 1,000 ml ราคา 209.00 บาท</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9zvDFSl7uu</t>
+          <t>https://s.shopee.co.th/8V6LwRFcsS</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134207-7rd5l-m70gtvlk15ck4a.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-lopnhfgn1k599e.webp</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -3115,17 +3109,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>BIO น้ำยาดับกลิ่น กลิ่นฉี่ กลิ่นมูลสัตว์เลี้ยง ล้างพื้นกลิ่นฉี่ ทำความสะอาด ปราศจากเชื้อโรค กลิ่นโอโซนบริสุทธิ์ 1,000 ml ราคา 209.00 บาท</t>
+          <t>ข้าวโพดบดละเอียด ขนาด 5 กก. ราคา 135.00 บาท</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8V6LwRFcsS</t>
+          <t>https://s.shopee.co.th/2LVm7GUCbl</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-lopnhfgn1k599e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98q-lr8as5tif5v2cf.webp</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -3136,21 +3130,21 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>10</v>
+        <v>126</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ข้าวโพดบดละเอียด ขนาด 5 กก. ราคา 135.00 บาท</t>
+          <t>[แบรนด์ขายดีอันดับ 1]JerHigh เจอร์ไฮ สติ๊ก ขนมสุนัข ขนาด 60 กรัม จำนวน 12 ซอง (เลือกรสด้านใน) ราคา 741.00 บาท</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2LVm7GUCbl</t>
+          <t>https://s.shopee.co.th/7VDsH33sg7</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98q-lr8as5tif5v2cf.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0s-mb7mtm884ks64b.webp</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -3161,46 +3155,46 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>126</v>
+        <v>62</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>[แบรนด์ขายดีอันดับ 1]JerHigh เจอร์ไฮ สติ๊ก ขนมสุนัข ขนาด 60 กรัม จำนวน 12 ซอง (เลือกรสด้านใน) ราคา 741.00 บาท</t>
+          <t>Dog Days อาหารสุนัขรสเนื้อแกะ (12 kg) Daily เกรด Holistic สูตรลดขนร่วงโดยเฉพาะ โซเดียมต่ำ ราคา 1691.00 บาท</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7VDsH33sg7</t>
+          <t>https://s.shopee.co.th/8fPpf2BSBB</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0s-mb7mtm884ks64b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mp3judrlwkcr9c.webp</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>done 2026-06-26 06:03</t>
+          <t>done 2026-06-27 05:50</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>62</v>
+        <v>93</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Dog Days อาหารสุนัขรสเนื้อแกะ (12 kg) Daily เกรด Holistic สูตรลดขนร่วงโดยเฉพาะ โซเดียมต่ำ ราคา 1691.00 บาท</t>
+          <t>PANDO Pet Smart Camera Feeder 4L เครื่องให้อาหารอัตโนมัติขนาด 4 ลิตร พร้อมกล้องวิดีโอ ราคา 3790.00 บาท</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8fPpf2BSBB</t>
+          <t>https://s.shopee.co.th/AUrTqTY04A</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mp3judrlwkcr9c.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mp20hqahb9xq74.webp</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -3211,21 +3205,21 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>93</v>
+        <v>128</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PANDO Pet Smart Camera Feeder 4L เครื่องให้อาหารอัตโนมัติขนาด 4 ลิตร พร้อมกล้องวิดีโอ ราคา 3790.00 บาท</t>
+          <t>Kasty Pop Tofu Litter ทรายแมวเต้าหู้ จับตัวเป็นก้อนเร็ว ทิ้งชักโครกได้ สำหรับแมวทุกวัย ราคา 160.00 บาท</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AUrTqTY04A</t>
+          <t>https://s.shopee.co.th/4ftgtqSxyR</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mp20hqahb9xq74.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mne6oge82upud0.webp</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -3236,21 +3230,21 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>128</v>
+        <v>38</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Kasty Pop Tofu Litter ทรายแมวเต้าหู้ จับตัวเป็นก้อนเร็ว ทิ้งชักโครกได้ สำหรับแมวทุกวัย ราคา 160.00 บาท</t>
+          <t>[ขายดี]สมาร์ทฮาร์ท อาหารสุนัข สุนัขโต รสไก่และตับ 10 กก. / SmartHeart Adult Chicken &amp; Liver 10kg ราคา 819.00 บาท</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4ftgtqSxyR</t>
+          <t>https://s.shopee.co.th/AKY3e27PbA</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mne6oge82upud0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m682t119n2yee3.webp</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -3261,71 +3255,71 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>[ขายดี]สมาร์ทฮาร์ท อาหารสุนัข สุนัขโต รสไก่และตับ 10 กก. / SmartHeart Adult Chicken &amp; Liver 10kg ราคา 819.00 บาท</t>
+          <t>[🔥6.6ลดสูงสุด450]My Paws กระบะทรายแบบจัมโบ้ ขนาด 64Cm กระบะทรายแมว ห้องน้ำแมวขนาดใหญ่ ราคา 234.00 บาท</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AKY3e27PbA</t>
+          <t>https://s.shopee.co.th/5L9Ngzmag2</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m682t119n2yee3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m2q2wkuxrsszbd.webp</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>done 2026-06-27 05:50</t>
+          <t>done 2026-06-27 05:51</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>[🔥6.6ลดสูงสุด450]My Paws กระบะทรายแบบจัมโบ้ ขนาด 64Cm กระบะทรายแมว ห้องน้ำแมวขนาดใหญ่ ราคา 234.00 บาท</t>
+          <t>MOMOVIDA CC-1 กระบะทรายแมวขนาดใหญ่ ห้องน้ำแมวขนาดใหญ่ ขอบสูงกันกระเด็น กระบะทรายจัมโบ้ มีที่ดักทราย กระบะทราย ราคา 639.00 บาท</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5L9Ngzmag2</t>
+          <t>https://s.shopee.co.th/3B4t6tK4Lg</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m2q2wkuxrsszbd.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-moz7fd2itb7lc0.webp</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>done 2026-06-27 05:51</t>
+          <t>done 2026-06-28 05:43</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>48</v>
+        <v>11</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>MOMOVIDA CC-1 กระบะทรายแมวขนาดใหญ่ ห้องน้ำแมวขนาดใหญ่ ขอบสูงกันกระเด็น กระบะทรายจัมโบ้ มีที่ดักทราย กระบะทราย ราคา 639.00 บาท</t>
+          <t>ไดร์เป่าขนสุนัข ขนแมว ขนหมา เครื่องเป่าขนสุนัข สัตว์เลี้ยง เสียงเงียบกว่าไดร์คน รุ่น MN-636 |Haftigt ราคา 2989.00 บาท</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3B4t6tK4Lg</t>
+          <t>https://s.shopee.co.th/gNY8CeoFf</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-moz7fd2itb7lc0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mo6m27kq42kl45.webp</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -3336,21 +3330,21 @@
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ไดร์เป่าขนสุนัข ขนแมว ขนหมา เครื่องเป่าขนสุนัข สัตว์เลี้ยง เสียงเงียบกว่าไดร์คน รุ่น MN-636 |Haftigt ราคา 2989.00 บาท</t>
+          <t>Prowild โปรไวลด์ ซีเล็คเต็ด อาหารสุนัขทุกสายพันธุ์/ทุกช่วงวัย ขนาด 15 kg ราคา 1590.00 บาท</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/gNY8CeoFf</t>
+          <t>https://s.shopee.co.th/9fIJKaWMHK</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mo6m27kq42kl45.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0m-mbg6gn8vi82g66.webp</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -3361,46 +3355,46 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Prowild โปรไวลด์ ซีเล็คเต็ด อาหารสุนัขทุกสายพันธุ์/ทุกช่วงวัย ขนาด 15 kg ราคา 1590.00 บาท</t>
+          <t>บ้านน็อคดาวน์ทรงโมเดิร์น ราคา 65000.00 บาท</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fIJKaWMHK</t>
+          <t>https://s.shopee.co.th/9AM6FuYLEz</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0m-mbg6gn8vi82g66.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-m87g7gynxs6me4.webp</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>done 2026-06-28 05:43</t>
+          <t>done 2026-06-28 05:44</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>บ้านน็อคดาวน์ทรงโมเดิร์น ราคา 65000.00 บาท</t>
+          <t>[ยกลัง 48 ซอง]Me o delite มีโอดีไลท์อาหารเปียกแมว ขนาด 70กรัม × 48 ซอง (มี 4 โหล) สินค้าพร้อมจัดส่ง ราคา 1109.00 บาท</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9AM6FuYLEz</t>
+          <t>https://s.shopee.co.th/8KmzGPHWgI</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-m87g7gynxs6me4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98o-lnk1fzypx3cg05.webp</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -3411,46 +3405,46 @@
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>[ยกลัง 48 ซอง]Me o delite มีโอดีไลท์อาหารเปียกแมว ขนาด 70กรัม × 48 ซอง (มี 4 โหล) สินค้าพร้อมจัดส่ง ราคา 1109.00 บาท</t>
+          <t>Prama อาหารสุนัขพราม่าเกรด Holistic มีให้เลือก 2 สูตร เนื้อแกะ และ ปลาทูน่า ขนาด 15kg ราคา 1250.00 บาท</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8KmzGPHWgI</t>
+          <t>https://s.shopee.co.th/9Uywec7H9V</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98o-lnk1fzypx3cg05.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m2idzdnzkn8k02.webp</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>done 2026-06-28 05:44</t>
+          <t>done 2026-06-29 05:43</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Prama อาหารสุนัขพราม่าเกรด Holistic มีให้เลือก 2 สูตร เนื้อแกะ และ ปลาทูน่า ขนาด 15kg ราคา 1250.00 บาท</t>
+          <t>บ้านน็อคดาวน์ สำเร็จรูป ราคา 150000.00 บาท</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9Uywec7H9V</t>
+          <t>https://s.shopee.co.th/30lPOKnQ4s</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m2idzdnzkn8k02.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m7wxzwgmmrgc2f.webp</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -3461,21 +3455,21 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>บ้านน็อคดาวน์ สำเร็จรูป ราคา 150000.00 บาท</t>
+          <t>Doge&amp;Orange ถุงมือเช็ดตัวสัตว์เลี้ยง ถุงมืออาบน้ำแมว สุนัข สูตรอ่อนโยน ไม่มีแอลกอฮอล์ ปลอดภัยกับสัตว์เลี้ยง PU165 ราคา 69.00 บาท</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/30lPOKnQ4s</t>
+          <t>https://s.shopee.co.th/110OWyMZpF</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m7wxzwgmmrgc2f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mm8mdlhwkav551.webp</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -3486,21 +3480,21 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Doge&amp;Orange ถุงมือเช็ดตัวสัตว์เลี้ยง ถุงมืออาบน้ำแมว สุนัข สูตรอ่อนโยน ไม่มีแอลกอฮอล์ ปลอดภัยกับสัตว์เลี้ยง PU165 ราคา 69.00 บาท</t>
+          <t>อ่างปลา บ่อบัว ขนาดใหญ่ (70cm/90cm/120cm) ราคา 2444.00 บาท</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/110OWyMZpF</t>
+          <t>https://s.shopee.co.th/3qKZu7RqK5</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mm8mdlhwkav551.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98y-lz61mc5dvfk1f7.webp</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -3511,96 +3505,96 @@
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>อ่างปลา บ่อบัว ขนาดใหญ่ (70cm/90cm/120cm) ราคา 2444.00 บาท</t>
+          <t>PANDO Pet Dryer Room PD65 แพนโด้ เครื่องเป่าขน สำหรับสัตว์เลี้ยง รุ่น PD65 ตู้เป่าขน อัตโนม ราคา 9990.00 บาท</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qKZu7RqK5</t>
+          <t>https://s.shopee.co.th/2qRzC0bKNG</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98y-lz61mc5dvfk1f7.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mp1zyxmcgm4r44.webp</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>done 2026-06-29 05:43</t>
+          <t>done 2026-06-29 05:44</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PANDO Pet Dryer Room PD65 แพนโด้ เครื่องเป่าขน สำหรับสัตว์เลี้ยง รุ่น PD65 ตู้เป่าขน อัตโนม ราคา 9990.00 บาท</t>
+          <t>Petoya คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุนัขและแมว สูตร Joint Focus + DHA ราคา 490.00 บาท</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qRzC0bKNG</t>
+          <t>https://s.shopee.co.th/6py7xOYUW1</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mp1zyxmcgm4r44.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lxa2x1xegij3c3.webp</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>done 2026-06-29 05:44</t>
+          <t>done 2026-06-30 05:40</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>19</v>
+        <v>107</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Petoya คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุนัขและแมว สูตร Joint Focus + DHA ราคา 490.00 บาท</t>
+          <t>yoyopet : แปรงกําจัดขนสองด้าน แปรงสางขนเสีย หวีซี่สแตนเลส กำจัดขนลอย ขนปม อุปกรณ์ดูแลขนสัตว์เลี้ยง ราคา 58.00 บาท</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6py7xOYUW1</t>
+          <t>https://s.shopee.co.th/7fXITJ3q7F</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lxa2x1xegij3c3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4ze403ouvtpc2.webp</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>done 2026-06-30 05:40</t>
+          <t>done 2026-06-30 05:41</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>yoyopet : แปรงกําจัดขนสองด้าน แปรงสางขนเสีย หวีซี่สแตนเลส กำจัดขนลอย ขนปม อุปกรณ์ดูแลขนสัตว์เลี้ยง ราคา 58.00 บาท</t>
+          <t>Pawdy อาหารสุนัขเกรดพรีเมียม สำหรับสุนัขสูงวัย อายุมากกว่า 7 ปี สูตรแกะและปลา ผสมเนื้อจระเข้ ขนาด 1.2 กก. (2 ถุง) ราคา 643.00 บาท</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7fXITJ3q7F</t>
+          <t>https://s.shopee.co.th/4qD763Stp2</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4ze403ouvtpc2.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mkgeybc3sfewa9.webp</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -3611,21 +3605,21 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>90</v>
+        <v>25</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Pawdy อาหารสุนัขเกรดพรีเมียม สำหรับสุนัขสูงวัย อายุมากกว่า 7 ปี สูตรแกะและปลา ผสมเนื้อจระเข้ ขนาด 1.2 กก. (2 ถุง) ราคา 643.00 บาท</t>
+          <t>Rojeco เครื ่ องป ้ อนแมวอัตโนมัติ 2L ปุ ่ ม/WIFI รุ ่ นควบคุมเครื ่ องป ้ อนอัตโนมัติสําหรับแมวสุนัขอุปกรณ ์ เสริม ราคา 960.00 บาท</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4qD763Stp2</t>
+          <t>https://s.shopee.co.th/60P4U2c3Lx</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mkgeybc3sfewa9.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-mlbstzaeel1dbf.webp</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -3636,21 +3630,21 @@
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Rojeco เครื ่ องป ้ อนแมวอัตโนมัติ 2L ปุ ่ ม/WIFI รุ ่ นควบคุมเครื ่ องป ้ อนอัตโนมัติสําหรับแมวสุนัขอุปกรณ ์ เสริม ราคา 960.00 บาท</t>
+          <t>สมาร์ทฮาร์ท โกลด์ ซีเลกต์ มูสลี่ กระต่าย 1.5 กิโลกรัม / SmartHeart Gold Zelect Muesli 1.5 KG ราคา 215.00 บาท</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/60P4U2c3Lx</t>
+          <t>https://s.shopee.co.th/5fmE5PH2YG</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-mlbstzaeel1dbf.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mmsjjqbyplol28.webp</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -3661,46 +3655,46 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>สมาร์ทฮาร์ท โกลด์ ซีเลกต์ มูสลี่ กระต่าย 1.5 กิโลกรัม / SmartHeart Gold Zelect Muesli 1.5 KG ราคา 215.00 บาท</t>
+          <t>KUMAま ห้องน้ำแมว Minimal Design ห้องน้ำใหญ่ แบบลิ้นชัก เก็บกลิ่น มินิมอลสไตล์ พร้อม แผ่นดักทราย &amp; ที่ตักทรายแมว ในเซ็ท ราคา 1050.00 บาท</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5fmE5PH2YG</t>
+          <t>https://s.shopee.co.th/3VhjVQCmD1</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mmsjjqbyplol28.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/95304806a08cb14f3f200cb4697e75f1.webp</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>done 2026-06-30 05:41</t>
+          <t>done 2026-07-01 05:57</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>KUMAま ห้องน้ำแมว Minimal Design ห้องน้ำใหญ่ แบบลิ้นชัก เก็บกลิ่น มินิมอลสไตล์ พร้อม แผ่นดักทราย &amp; ที่ตักทรายแมว ในเซ็ท ราคา 1050.00 บาท</t>
+          <t>เสื้อจุดให้สัตว์เลี้ยง เสื้อแมว เสื้อผ้าสัตว์เลี้ยง เดรสสายเดี่ยว น่ารักมาก ระบายอากาศ Sweet girl style ราคา 51.00 บาท</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3VhjVQCmD1</t>
+          <t>https://s.shopee.co.th/80A8rsR9jI</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/95304806a08cb14f3f200cb4697e75f1.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-824is-mfnt7nm8oufefe.webp</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -3711,21 +3705,21 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>91</v>
+        <v>24</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>เสื้อจุดให้สัตว์เลี้ยง เสื้อแมว เสื้อผ้าสัตว์เลี้ยง เดรสสายเดี่ยว น่ารักมาก ระบายอากาศ Sweet girl style ราคา 51.00 บาท</t>
+          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology ทรายแมวภูเขาไฟ เก็บกลิ่นดี ไม่มีฝุ่น จับตัวไว ปลอดภัยต่อคนและสัตว์เลี้ยง Sand Here ราคา 510.00 บาท</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/80A8rsR9jI</t>
+          <t>https://s.shopee.co.th/6felHGQZub</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-824is-mfnt7nm8oufefe.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0p-mbdqsabjn29i2f.webp</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -3736,21 +3730,21 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>24</v>
+        <v>117</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology ทรายแมวภูเขาไฟ เก็บกลิ่นดี ไม่มีฝุ่น จับตัวไว ปลอดภัยต่อคนและสัตว์เลี้ยง Sand Here ราคา 510.00 บาท</t>
+          <t>PANDO Double-Layer Pet Trolley แพนโด้ รถเข็นแบบสองชั้นสำหรับสัตว์เลี้ยง ราคา 5990.00 บาท</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6felHGQZub</t>
+          <t>https://s.shopee.co.th/40e06ahvjJ</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0p-mbdqsabjn29i2f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mj6sg1hg00sj92.webp</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -3761,21 +3755,21 @@
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>117</v>
+        <v>27</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>PANDO Double-Layer Pet Trolley แพนโด้ รถเข็นแบบสองชั้นสำหรับสัตว์เลี้ยง ราคา 5990.00 บาท</t>
+          <t>คอลลาเจนญี่ปุ่นบำรุงขนและข้อสำหรับสุนัขแมว สูตรแพ้ง่าย แพ้ไก่ แพ้อาหารทะเลทานได้ ราคา 456.00 บาท</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/40e06ahvjJ</t>
+          <t>https://s.shopee.co.th/2LVm7J6mm7</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mj6sg1hg00sj92.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98r-lxa2x1xegib446.webp</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -3786,46 +3780,46 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>คอลลาเจนญี่ปุ่นบำรุงขนและข้อสำหรับสุนัขแมว สูตรแพ้ง่าย แพ้ไก่ แพ้อาหารทะเลทานได้ ราคา 456.00 บาท</t>
+          <t>[Doctor By BREATH CARE] อาหารเสริมทางเดินหายใจสุนัข บรรเทาอาการไอ ฮอนคิง แก้สงสารพยุงบรอนเชียล (30 บีบ) ราคา 1126.00 บาท</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2LVm7J6mm7</t>
+          <t>https://s.shopee.co.th/8KmzGMOid3</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98r-lxa2x1xegib446.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134207-822wp-mog5oph3ouml25.webp</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>done 2026-07-01 05:57</t>
+          <t>done 2026-07-02 05:52</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>[Doctor By BREATH CARE] อาหารเสริมทางเดินหายใจสุนัข บรรเทาอาการไอ ฮอนคิง แก้สงสารพยุงบรอนเชียล (30 บีบ) ราคา 1126.00 บาท</t>
+          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK V.3 และ CATLINK V.3 Ultra ราคา 13900.00 บาท</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8KmzGMOid3</t>
+          <t>https://s.shopee.co.th/5fmAZDqFhJ</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134207-822wp-mog5oph3ouml25.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0k-mbdr25xh8y299a.webp</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -3836,21 +3830,21 @@
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>6</v>
+        <v>105</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>[🔥ใส่โค้ดลดเพิ่ม] Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK V.3 และ CATLINK V.3 Ultra ราคา 13900.00 บาท</t>
+          <t>โต๊ะวางชามอาหารน้องแมว และ น้องหมา น่ารัก Minimal + พร้อมถ้วย ราคา 199.00 บาท</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5fmAZDqFhJ</t>
+          <t>https://s.shopee.co.th/5ApxUhwVwS</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0k-mbdr25xh8y299a.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7quky-lfr5jol6j09b5d.webp</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -3861,21 +3855,21 @@
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>105</v>
+        <v>47</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>โต๊ะวางชามอาหารน้องแมว และ น้องหมา น่ารัก Minimal + พร้อมถ้วย ราคา 199.00 บาท</t>
+          <t>[ชุดสุดคุ้ม]FRONTLINE PLUS CAT ผลิตภัณฑ์หยดกำจัดเห็บหมัด สำหรับแมว (จำนวน 2 กล่อง 6 หลอด) ราคา 982.00 บาท</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5ApxUhwVwS</t>
+          <t>https://s.shopee.co.th/6pyBTczAQp</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7quky-lfr5jol6j09b5d.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasl-m9fm7cscxs9s76.webp</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -3886,71 +3880,71 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>[ชุดสุดคุ้ม]FRONTLINE PLUS CAT ผลิตภัณฑ์หยดกำจัดเห็บหมัด สำหรับแมว (จำนวน 2 กล่อง 6 หลอด) ราคา 982.00 บาท</t>
+          <t>ขนมแมวเลีย มีโอ ขนมแมวเลีย เพอร์เฟคมิกซ์ ขนาด 1,500 กรัม (1 กล่อง 100 ซอง) ราคา 760.00 บาท</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6pyBTczAQp</t>
+          <t>https://s.shopee.co.th/40e06PQEmh</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasl-m9fm7cscxs9s76.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/abbb3e4423980f5077c3f5c9d1a5d9a0.webp</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>done 2026-07-02 05:52</t>
+          <t>done 2026-07-02 05:53</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>ขนมแมวเลีย มีโอ ขนมแมวเลีย เพอร์เฟคมิกซ์ ขนาด 1,500 กรัม (1 กล่อง 100 ซอง) ราคา 760.00 บาท</t>
+          <t>[15g x 30 ซอง] VetOLOGY ขนมเลียสำหรับแมวและสุนัข เหมาะกับทุกช่วงวัย ราคา 368.00 บาท</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/40e06PQEmh</t>
+          <t>https://s.shopee.co.th/gNY8OEigK</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/abbb3e4423980f5077c3f5c9d1a5d9a0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasg-m8vl08x42lhree.webp</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>done 2026-07-02 05:53</t>
+          <t>done 2026-07-03 05:47</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>[15g x 30 ซอง] VetOLOGY ขนมเลียสำหรับแมวและสุนัข เหมาะกับทุกช่วงวัย ราคา 368.00 บาท</t>
+          <t>I&amp;CATอพาร์ทเมนท์แมว ผ้ากำมะหยี่ 2 ชั้น ลับเล็บ เล่น นอน เสาเชือกปอหนา บ้านแมว เตียงแมว แข็งแรงมั่นคง ราคา 299.00 บาท</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/gNY8OEigK</t>
+          <t>https://s.shopee.co.th/6pyBTmPzBM</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasg-m8vl08x42lhree.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-8262h-mk28fdijuvwj73.webp</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -3961,21 +3955,21 @@
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>109</v>
+        <v>36</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>I&amp;CATอพาร์ทเมนท์แมว ผ้ากำมะหยี่ 2 ชั้น ลับเล็บ เล่น นอน เสาเชือกปอหนา บ้านแมว เตียงแมว แข็งแรงมั่นคง ราคา 299.00 บาท</t>
+          <t>Cutepol ทรายแมวเต้าหู้ ดับกลิ่นสูงสุด จับตัวก้อนแน่น แบบผสม หลายขนาด (35L/21L/7L) | Mixed Cat Litter ราคา 499.00 บาท</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6pyBTmPzBM</t>
+          <t>https://s.shopee.co.th/5VSnt9891q</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-8262h-mk28fdijuvwj73.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-moz7ekcbezuqaa.webp</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -3986,21 +3980,21 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Cutepol ทรายแมวเต้าหู้ ดับกลิ่นสูงสุด จับตัวก้อนแน่น แบบผสม หลายขนาด (35L/21L/7L) | Mixed Cat Litter ราคา 499.00 บาท</t>
+          <t>🏆Pupping Petmat รุ่น Rug Type M - L แผ่นกันลื่นสุนัข พรมกันลื่น รองกันลื่นสัตว์เลี้ยง หมาแมว ป้องกันข้อสะโพกเสื่อม 🇰🇷 ราคา 4250.00 บาท</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5VSnt9891q</t>
+          <t>https://s.shopee.co.th/4LGqV4sgyW</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-moz7ekcbezuqaa.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98w-lygolxsp1g8xcf.webp</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -4011,21 +4005,21 @@
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>🏆Pupping Petmat รุ่น Rug Type M - L แผ่นกันลื่นสุนัข พรมกันลื่น รองกันลื่นสัตว์เลี้ยง หมาแมว ป้องกันข้อสะโพกเสื่อม 🇰🇷 ราคา 4250.00 บาท</t>
+          <t>สมาร์ทฮาร์ท อาหารสุนัข สำหรับลูกสุนัข รสเนื้อวัวและนม 15กก. ราคา 1030.00 บาท</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4LGqV4sgyW</t>
+          <t>https://s.shopee.co.th/gNY8RukUK</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98w-lygolxsp1g8xcf.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/9ec893796776a5020ab0abee60620b57.webp</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -4036,46 +4030,46 @@
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>110</v>
+        <v>26</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>สมาร์ทฮาร์ท อาหารสุนัข สำหรับลูกสุนัข รสเนื้อวัวและนม 15กก. ราคา 1030.00 บาท</t>
+          <t>Pawdy อาหารสุนัขเกรดพรีเมียม Holistic สำหรับสุนัขโต อายุ 1-6 ปี สูตรเนื้อแกะรมควัน ขนาด 8 กก. ราคา 1359.00 บาท</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/gNY8RukUK</t>
+          <t>https://s.shopee.co.th/9pbn35XQb1</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/9ec893796776a5020ab0abee60620b57.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mn700alam03s8d.webp</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>done 2026-07-03 05:47</t>
+          <t>done 2026-07-04 05:42</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Pawdy อาหารสุนัขเกรดพรีเมียม Holistic สำหรับสุนัขโต อายุ 1-6 ปี สูตรเนื้อแกะรมควัน ขนาด 8 กก. ราคา 1359.00 บาท</t>
+          <t>Virbac น้ำยาทำความสะอาดช่องหู อิพิโอติก [EpiOtic® Ear Cleaning - 125ml] สูตรไมเซลลาร์ สำหรับสุนัขและแมว ทุกช่วงวัย ราคา 493.00 บาท</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9pbn35XQb1</t>
+          <t>https://s.shopee.co.th/4qD75qVfyK</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mn700alam03s8d.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasf-m2rp6pad7j2kfb.webp</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -4086,21 +4080,21 @@
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Virbac น้ำยาทำความสะอาดช่องหู อิพิโอติก [EpiOtic® Ear Cleaning - 125ml] สูตรไมเซลลาร์ สำหรับสุนัขและแมว ทุกช่วงวัย ราคา 493.00 บาท</t>
+          <t>12 แพ็ค (48 ซอง) CATE เคท ขนมแมวเลีย คอลลาเจน พรีไบโอติก เสริมภูมิ แคลเซียม ราคา 639.00 บาท</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4qD75qVfyK</t>
+          <t>https://s.shopee.co.th/7VDsGoDaFN</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasf-m2rp6pad7j2kfb.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mowokonm6xam07.webp</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -4111,21 +4105,21 @@
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>30</v>
+        <v>88</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>12 แพ็ค (48 ซอง) CATE เคท ขนมแมวเลีย คอลลาเจน พรีไบโอติก เสริมภูมิ แคลเซียม ราคา 639.00 บาท</t>
+          <t>FABLEME —PET BASKET เข่งใส่แมว ตระกร้าที่นอนแมวแบบเข่ง สไตล์มินิมอลง ราคา 200.00 บาท</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7VDsGoDaFN</t>
+          <t>https://s.shopee.co.th/9zvDFXsO5l</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mowokonm6xam07.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mnrcaodqhb0k02.webp</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -4136,21 +4130,21 @@
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>88</v>
+        <v>23</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>FABLEME —PET BASKET เข่งใส่แมว ตระกร้าที่นอนแมวแบบเข่ง สไตล์มินิมอลง ราคา 200.00 บาท</t>
+          <t>[สินค้าใหม่] PANDO Pet Hair Trimmer 4 in 1 Pro แพนโด้ ชุดอุปกรณ์ตัดขน เล็มขน สัตว์เลี้ยง รุ่น โปร ราคา 581.00 บาท</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9zvDFXsO5l</t>
+          <t>https://s.shopee.co.th/30lSuWWyVO</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mnrcaodqhb0k02.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mp20bnax2bkd6b.webp</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -4161,46 +4155,46 @@
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>[สินค้าใหม่] PANDO Pet Hair Trimmer 4 in 1 Pro แพนโด้ ชุดอุปกรณ์ตัดขน เล็มขน สัตว์เลี้ยง รุ่น โปร ราคา 581.00 บาท</t>
+          <t>ทรายแมว แคสตี้ Kasty ทรายแมวเต้าหู้ ธรรมชาติ ดับกลิ่นดีเยี่ยม จับตัวเป็นก้อนเร็ว 3 วินาที ขนาด 6 ลิตร ราคา 230.00 บาท</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/30lSuWWyVO</t>
+          <t>https://s.shopee.co.th/1BJojJz0UM</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mp20bnax2bkd6b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98q-lv44o0d5n8c399.webp</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>done 2026-07-04 05:42</t>
+          <t>done 2026-07-05 05:39</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>92</v>
+        <v>33</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>ทรายแมว แคสตี้ Kasty ทรายแมวเต้าหู้ ธรรมชาติ ดับกลิ่นดีเยี่ยม จับตัวเป็นก้อนเร็ว 3 วินาที ขนาด 6 ลิตร ราคา 230.00 บาท</t>
+          <t>😺 สินค้าอยู่ในไทย พร้อมส่ง 🐱 กรงแมว กรงขังแมว Pet Cage วิลล่าแมวไม้ กรงเเมวอพาร์ทเมนต์แมวไม้เนื้อแข็ง บ้านแมวขนาดใหญ่ ราคา 1698.00 บาท</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1BJojJz0UM</t>
+          <t>https://s.shopee.co.th/1LdEvTx3g8</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98q-lv44o0d5n8c399.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qukw-ljnz6fkjjebt84.webp</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -4211,21 +4205,21 @@
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>33</v>
+        <v>114</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>😺 สินค้าอยู่ในไทย พร้อมส่ง 🐱 กรงแมว กรงขังแมว Pet Cage วิลล่าแมวไม้ กรงเเมวอพาร์ทเมนต์แมวไม้เนื้อแข็ง บ้านแมวขนาดใหญ่ ราคา 1698.00 บาท</t>
+          <t>(คละรสไม่ได้) สมาร์ทฮาร์ท อาหารสุนัขกระป๋อง 400g x24 กระป๋อง(ยกแพ็ค) ราคา 1090.00 บาท</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1LdEvTx3g8</t>
+          <t>https://s.shopee.co.th/9KfWSNx5gi</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qukw-ljnz6fkjjebt84.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mlx53j8akmbp86.webp</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -4236,46 +4230,46 @@
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>114</v>
+        <v>14</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>(คละรสไม่ได้) สมาร์ทฮาร์ท อาหารสุนัขกระป๋อง 400g x24 กระป๋อง(ยกแพ็ค) ราคา 1090.00 บาท</t>
+          <t>Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK Lite ราคา 8800.00 บาท</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9KfWSNx5gi</t>
+          <t>https://s.shopee.co.th/60P0xquu84</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mlx53j8akmbp86.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-mauvmoz6b0omd5.webp</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>done 2026-07-05 05:39</t>
+          <t>done 2026-07-05 05:40</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK Lite ราคา 8800.00 บาท</t>
+          <t>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์ ราคา 547.00 บาท</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/60P0xquu84</t>
+          <t>https://s.shopee.co.th/W47vxAxHm</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-mauvmoz6b0omd5.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -4286,46 +4280,46 @@
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>34</v>
+        <v>96</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์ ราคา 547.00 บาท</t>
+          <t>🔥【PET RECORD】กระบะทรายแมวขนาดใหญ่ ขอบสูง ป้องกันทรายกระเด็น ห้องน้ำแมวฝาปิดถอดล้างง่าย แข็งแรง ทนทาน ราคา 52.00 บาท</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/W47vxAxHm</t>
+          <t>https://s.shopee.co.th/8fPpf75rJi</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mh8j9ug03or2f9.webp</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>done 2026-07-05 05:40</t>
+          <t>done 2026-07-06 05:40</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>🔥【PET RECORD】กระบะทรายแมวขนาดใหญ่ ขอบสูง ป้องกันทรายกระเด็น ห้องน้ำแมวฝาปิดถอดล้างง่าย แข็งแรง ทนทาน ราคา 52.00 บาท</t>
+          <t>🐈🐱Neakasa M1 2024 ห้องน้ำแมวอัตโนมัติ I Smart Cat Litter I จัดการข้อมูลแมว 3 ตัว I แอปควบคุมระยะไกล🐈🐱 ราคา 10499.00 บาท</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8fPpf75rJi</t>
+          <t>https://s.shopee.co.th/8V6LwSP3Kc</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mh8j9ug03or2f9.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasi-m6oxwve9ydkf40.webp</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -4336,21 +4330,21 @@
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>18</v>
+        <v>127</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>🐈🐱Neakasa M1 2024 ห้องน้ำแมวอัตโนมัติ I Smart Cat Litter I จัดการข้อมูลแมว 3 ตัว I แอปควบคุมระยะไกล🐈🐱 ราคา 10499.00 บาท</t>
+          <t>【30 ชิ้นในแพ็คเกจใหญ่】📍 ลูกกลิ้งกำจัดขน เก็บขนและฝุ่น ลูกกลิ้งทำความสะอาด ลูกกลิ้งเก็บฝุ่น ลูกกลิ้งดักฝุ่น ที่เก็บขน ราคา 60.00 บาท</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8V6LwSP3Kc</t>
+          <t>https://s.shopee.co.th/3VhjVhT0YU</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasi-m6oxwve9ydkf40.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zti-me9k1abrgzr7e3.webp</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -4361,21 +4355,21 @@
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>127</v>
+        <v>4</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>【30 ชิ้นในแพ็คเกจใหญ่】📍 ลูกกลิ้งกำจัดขน เก็บขนและฝุ่น ลูกกลิ้งทำความสะอาด ลูกกลิ้งเก็บฝุ่น ลูกกลิ้งดักฝุ่น ที่เก็บขน ราคา 60.00 บาท</t>
+          <t>F&amp;G วิลล่าแมว Cat Villa บ้านแมว กรงแมว วิลล่าไม้เนื้อแข็งตู้แมว ตู้โชว์ไม้เนื้อแข็ง วิลล่าแมวขนาดใหญ จัดส่งภายใน24ชั่วโม ราคา 1999.00 บาท</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3VhjVhT0YU</t>
+          <t>https://s.shopee.co.th/AAEZvUHexi</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zti-me9k1abrgzr7e3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m3ytl0pibu8a95.webp</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -4386,71 +4380,71 @@
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>F&amp;G วิลล่าแมว Cat Villa บ้านแมว กรงแมว วิลล่าไม้เนื้อแข็งตู้แมว ตู้โชว์ไม้เนื้อแข็ง วิลล่าแมวขนาดใหญ จัดส่งภายใน24ชั่วโม ราคา 1999.00 บาท</t>
+          <t>❤️ พร้อมส่ง แถมฝาปิด ส่งฟรี❤️ โอ่งแมวดินเผา16 18 20 นิ้ว บ้านแอร์แมว ราคา 692.00 บาท</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AAEZvUHexi</t>
+          <t>https://s.shopee.co.th/6felHDaFIV</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m3ytl0pibu8a95.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-23010-6v8kphz6xnmvbf.webp</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>done 2026-07-06 05:40</t>
+          <t>done 2026-07-06 05:41</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>❤️ พร้อมส่ง แถมฝาปิด ส่งฟรี❤️ โอ่งแมวดินเผา16 18 20 นิ้ว บ้านแอร์แมว ราคา 692.00 บาท</t>
+          <t>คอนโดแมว คอนโดแมวไม้ บ้านแมว เหมาะสำหรับเลี้ยงน้องแมว 4-6ตัว เสาลับเล็บ ขนาดใหญ่ สูง170CM ราคา 658.00 บาท</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6felHDaFIV</t>
+          <t>https://s.shopee.co.th/2qS2iMyQbg</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-23010-6v8kphz6xnmvbf.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-ml7kqp8bdwcic1.webp</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>done 2026-07-06 05:41</t>
+          <t>done 2026-07-07 05:47</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>85</v>
+        <v>19</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>คอนโดแมว คอนโดแมวไม้ บ้านแมว เหมาะสำหรับเลี้ยงน้องแมว 4-6ตัว เสาลับเล็บ ขนาดใหญ่ สูง170CM ราคา 658.00 บาท</t>
+          <t>Petoya คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุนัขและแมว สูตร Joint Focus + DHA ราคา 490.00 บาท</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qS2iMyQbg</t>
+          <t>https://s.shopee.co.th/3LOJJ7d3MA</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-ml7kqp8bdwcic1.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lxa2x1xegij3c3.webp</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -4461,21 +4455,21 @@
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Petoya คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุนัขและแมว สูตร Joint Focus + DHA ราคา 490.00 บาท</t>
+          <t>Dog Days อาหารลูกสุนัข (6 kg) สูตร Puppy &amp; Mommy รสแกะและปลาทูน่า ราคา 690.00 บาท</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3LOJJ7d3MA</t>
+          <t>https://s.shopee.co.th/110OWujz86</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lxa2x1xegij3c3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-modfibxbvymma0.webp</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -4486,439 +4480,414 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>50</v>
+        <v>131</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Dog Days อาหารลูกสุนัข (6 kg) สูตร Puppy &amp; Mommy รสแกะและปลาทูน่า ราคา 690.00 บาท</t>
+          <t>ยกโหล Nekko อาหารเปียกแมว 70 กรัม12ซอง</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/110OWujz86</t>
+          <t>https://s.shopee.co.th/1BJb9Qw4hN</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-modfibxbvymma0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mofbqutr8kcu6a.webp</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>฿159</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>done 2026-07-07 05:47</t>
+          <t>done 2026-07-16 22:01</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>ยกโหล Nekko อาหารเปียกแมว 70 กรัม12ซอง</t>
+          <t>FABLEME —PET BASKET เข่งใส่แมว ตระกร้าที่นอนแมวแบบเข่ง สไตล์มินิมอลง</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1BJb9Qw4hN</t>
+          <t>https://s.shopee.co.th/3B4fX6y9c8</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mofbqutr8kcu6a.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mnrcaodqhb0k02.webp</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>฿159</t>
+          <t>฿220</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>done 2026-07-16 22:01</t>
+          <t>done 2026-07-17 08:23</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>FABLEME —PET BASKET เข่งใส่แมว ตระกร้าที่นอนแมวแบบเข่ง สไตล์มินิมอลง</t>
+          <t>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3B4fX6y9c8</t>
+          <t>https://s.shopee.co.th/4AxCiwxzUR</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mnrcaodqhb0k02.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mhh7zikraarne4.webp</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>฿220</t>
+          <t>฿210</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>done 2026-07-17 08:23</t>
+          <t>done 2026-07-17 19:48</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม</t>
+          <t>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4AxCiwxzUR</t>
+          <t>https://s.shopee.co.th/2BC8LHMRmu</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mhh7zikraarne4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>฿210</t>
-        </is>
-      </c>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>done 2026-07-17 19:48</t>
+          <t>฿542</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์</t>
+          <t>[ประกันศูนย์ไทย] Oneisall Pet Grooming Vacuum Kit 8 in 1 ตัดขนแมว เครื่องดูดขนแมว ไดร์เป่าขนสุนัข ขนาด2.5L รุ่น BM1</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2BC8LHMRmu</t>
+          <t>https://s.shopee.co.th/3LO5jQQjkG</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0h-mdtub2gcu0oe50.webp</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>฿542</t>
+          <t>฿5212</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>[ประกันศูนย์ไทย] Oneisall Pet Grooming Vacuum Kit 8 in 1 ตัดขนแมว เครื่องดูดขนแมว ไดร์เป่าขนสุนัข ขนาด2.5L รุ่น BM1</t>
+          <t>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3LO5jQQjkG</t>
+          <t>https://s.shopee.co.th/qgkkpnnSC</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0h-mdtub2gcu0oe50.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>฿5212</t>
+          <t>฿7888</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI</t>
+          <t>((12ซอง คละรสได้)) Pramy พรามี่ อาหารเปียกแมว หลากหลายรส ขนาด 70g. สูตรลูกแมว แมวโต แมวสูงวัย</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/qgkkpnnSC</t>
+          <t>https://s.shopee.co.th/8KmlgcYJ3j</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mob33vjgv0gee0.webp</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>฿7888</t>
+          <t>฿265</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>((12ซอง คละรสได้)) Pramy พรามี่ อาหารเปียกแมว หลากหลายรส ขนาด 70g. สูตรลูกแมว แมวโต แมวสูงวัย</t>
+          <t>PANDO Pet Dryer Room PD65 แพนโด้ เครื่องเป่าขน สำหรับสัตว์เลี้ยง รุ่น PD65 ตู้เป่าขน อัตโนม</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8KmlgcYJ3j</t>
+          <t>https://s.shopee.co.th/6L1hIwoeQ7</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mob33vjgv0gee0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mojgkgp81dsf9b.webp</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>฿265</t>
+          <t>฿9990</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>PANDO Pet Dryer Room PD65 แพนโด้ เครื่องเป่าขน สำหรับสัตว์เลี้ยง รุ่น PD65 ตู้เป่าขน อัตโนม</t>
+          <t>ห้องน้ำแมวอัจฉริยะ ห้องน้ําแมวอัตโนมัติสามารถเก็บอุจจาระได้โดยอัตโนมัติตามการขับถ่ายของแมว หลีกเลี่ยงกลิ่นแปลก ๆ และยับย</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6L1hIwoeQ7</t>
+          <t>https://s.shopee.co.th/20si8zFjb6</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mojgkgp81dsf9b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mkf3obhghekg6a.webp</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>฿9990</t>
+          <t>฿3199</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>ห้องน้ำแมวอัจฉริยะ ห้องน้ําแมวอัตโนมัติสามารถเก็บอุจจาระได้โดยอัตโนมัติตามการขับถ่ายของแมว หลีกเลี่ยงกลิ่นแปลก ๆ และยับย</t>
+          <t>กล่องเดินทางสัตว์เลี้ยง กรงหิ้วแมว กรงเดินทาง กล่องใส่สัตว์เลี้ยง กรงเดินทาง กล่องใส่สัตว์เลี้ยง</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/20si8zFjb6</t>
+          <t>https://s.shopee.co.th/BR3xcUYD6</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mkf3obhghekg6a.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0g-mbm7xxs7he1kb4.webp</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>฿3199</t>
+          <t>฿973</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>กล่องเดินทางสัตว์เลี้ยง กรงหิ้วแมว กรงเดินทาง กล่องใส่สัตว์เลี้ยง กรงเดินทาง กล่องใส่สัตว์เลี้ยง</t>
+          <t>Pramy in Gravy 70g อาหารเปียกแมว แมวโต เกรวี่ 12ซอง สำหรับแมว2เดือนขึ้นไป Petus Kingkaew</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/BR3xcUYD6</t>
+          <t>https://s.shopee.co.th/2BC8LIUqJB</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0g-mbm7xxs7he1kb4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mornhzyf1w5qc6.webp</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>฿973</t>
+          <t>฿256</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Pramy in Gravy 70g อาหารเปียกแมว แมวโต เกรวี่ 12ซอง สำหรับแมว2เดือนขึ้นไป Petus Kingkaew</t>
+          <t>navipet Smart Pet Dryer (Thai Version) ตู้เป่า ขนสัตว์เลี้ยง 72ลิตร O ZONE ฆ่าเชื้อได้ ประกันศูนย์ไทย</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2BC8LIUqJB</t>
+          <t>https://s.shopee.co.th/LkU9vkgr8</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mornhzyf1w5qc6.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mnqj2jpnw45hd8.webp</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>฿256</t>
+          <t>฿7900</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>navipet Smart Pet Dryer (Thai Version) ตู้เป่า ขนสัตว์เลี้ยง 72ลิตร O ZONE ฆ่าเชื้อได้ ประกันศูนย์ไทย</t>
+          <t>ห้องน้ำแมวใหญ่ SMART CAT LITTER BO</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/LkU9vkgr8</t>
+          <t>https://s.shopee.co.th/7VDeh6StVB</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mnqj2jpnw45hd8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-822yl-mhwpnsjh6k1wff.webp</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>฿7900</t>
+          <t>฿1000</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>ห้องน้ำแมวใหญ่ SMART CAT LITTER BO</t>
+          <t>ขนมแมวเลีย Me-O มีโอ 11 รสชาติ คละรสได้ 11/20/25/36 ซอง | ขนมแมว อาหารแมวเลีย อาหารเสริมแมว</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7VDeh6StVB</t>
+          <t>https://s.shopee.co.th/1gFrkO6YwY</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-822yl-mhwpnsjh6k1wff.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mnyj1j3uxe6ad5.webp</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>฿1000</t>
+          <t>฿109</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>ขนมแมวเลีย Me-O มีโอ 11 รสชาติ คละรสได้ 11/20/25/36 ซอง | ขนมแมว อาหารแมวเลีย อาหารเสริมแมว</t>
+          <t>สเปรย์น้ำหอมระงับกลิ่น แบรนด์พราวพาว สูตรอ่อนโยน สารสกัดจากธรรมชาติ 3 กลิ่น หอมละมุนชื่นใจ</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1gFrkO6YwY</t>
+          <t>https://s.shopee.co.th/17dlKLdcu</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mnyj1j3uxe6ad5.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m2usz5kign3644.webp</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>฿109</t>
+          <t>฿169</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>สเปรย์น้ำหอมระงับกลิ่น แบรนด์พราวพาว สูตรอ่อนโยน สารสกัดจากธรรมชาติ 3 กลิ่น หอมละมุนชื่นใจ</t>
+          <t>กรงไก่กลางแจ้ง คอกไก่ บ้านไก่ ขนาดใหญ่พิเศษ สำหรับการเลี้ยงสัตว์ปีก กันฝน กรงนกยูงและนกพิราบ โครงสร้างขนาดใหญ่</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/17dlKLdcu</t>
+          <t>https://s.shopee.co.th/9Uyj4mysUr</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m2usz5kign3644.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mkdbuy6rdgjr2e.webp</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
-        <is>
-          <t>฿169</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="n">
-        <v>146</v>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>กรงไก่กลางแจ้ง คอกไก่ บ้านไก่ ขนาดใหญ่พิเศษ สำหรับการเลี้ยงสัตว์ปีก กันฝน กรงนกยูงและนกพิราบ โครงสร้างขนาดใหญ่</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/9Uyj4mysUr</t>
-        </is>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mkdbuy6rdgjr2e.webp</t>
-        </is>
-      </c>
-      <c r="F174" t="inlineStr">
         <is>
           <t>฿1224</t>
         </is>

</xml_diff>

<commit_message>
chore: resolve binary xlsx conflict from stash pop
</commit_message>
<xml_diff>
--- a/review_products.xlsx
+++ b/review_products.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="630" yWindow="615" windowWidth="37095" windowHeight="17310" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -642,11 +642,6 @@
           <t>https://s.shopee.co.th/3qKMKMpn2h</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://s.lazada.co.th/s.Z6mEyG?c=a&amp;t=p-i0-s0&amp;sub_id1=W1</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m3ytl0pibu8a95.webp</t>
@@ -4567,11 +4562,6 @@
           <t>฿210</t>
         </is>
       </c>
-      <c r="G160" t="inlineStr">
-        <is>
-          <t>done 2026-07-17 19:48</t>
-        </is>
-      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -4595,11 +4585,6 @@
       <c r="F161" t="inlineStr">
         <is>
           <t>฿542</t>
-        </is>
-      </c>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>done 2026-07-18 19:38</t>
         </is>
       </c>
     </row>
@@ -4928,7 +4913,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>{"last_personas": ["F", "E", "C", "H", "C", "G", "F", "A", "G", "E", "C", "C", "H", "E", "D", "C", "H", "F", "E", "F", "B", "E", "E", "F", "B", "E", "H", "D", "C", "H", "G", "G", "D", "A", "F", "H", "F", "G", "D", "A", "G", "A", "F", "F", "A", "H", "F", "G", "E", "H"], "last_hooks": ["เห็นคนพูดถึงเยอะเลยลอง", "มีใครเป็นเหมือนผมไหม", "อันนี้เกินคาดจริงๆ", "เมื่อวานเพิ่งเจอ...", "ตอนแรกไม่ได้จะซื้อ", "กำลังหาของแบบนี้อยู่พอดี", "แชร์เผื่อมีคนกำลังหาอยู่", "โดนป้ายยามาอีกที", "ไม่คิดว่าจะ...", "ลองแล้วเข้าใจเลยว่าทำไมขายดี", "เห็นคนพูดถึงเยอะเลยลอง", "มีใครเป็นเหมือนผมไหม", "อันนี้เกินคาดจริงๆ", "เมื่อวานเพิ่งเจอ...", "ตอนแรกไม่ได้จะซื้อ", "กำลังหาของแบบนี้อยู่พอดี", "แชร์เผื่อมีคนกำลังหาอยู่", "โดนป้ายยามาอีกที", "ไม่คิดว่าจะ...", "ลองแล้วเข้าใจเลยว่าทำไมขายดี", "เห็นคนพูดถึงเยอะเลยลอง", "มีใครเป็นเหมือนผมไหม", "อันนี้เกินคาดจริงๆ", "เมื่อวานเพิ่งเจอ...", "ตอนแรกไม่ได้จะซื้อ", "กำลังหาของแบบนี้อยู่พอดี", "แชร์เผื่อมีคนกำลังหาอยู่", "โดนป้ายยามาอีกที", "ไม่คิดว่าจะ...", "ลองแล้วเข้าใจเลยว่าทำไมขายดี", "เห็นคนพูดถึงเยอะเลยลอง", "มีใครเป็นเหมือนผมไหม", "อันนี้เกินคาดจริงๆ", "เมื่อวานเพิ่งเจอ...", "ตอนแรกไม่ได้จะซื้อ", "กำลังหาของแบบนี้อยู่พอดี", "แชร์เผื่อมีคนกำลังหาอยู่", "โดนป้ายยามาอีกที", "ไม่คิดว่าจะ...", "ลองแล้วเข้าใจเลยว่าทำไมขายดี", "เห็นคนพูดถึงเยอะเลยลอง", "มีใครเป็นเหมือนผมไหม", "อันนี้เกินคาดจริงๆ", "เมื่อวานเพิ่งเจอ...", "ตอนแรกไม่ได้จะซื้อ", "กำลังหาของแบบนี้อยู่พอดี", "แชร์เผื่อมีคนกำลังหาอยู่", "โดนป้ายยามาอีกที", "ไม่คิดว่าจะ...", "ลองแล้วเข้าใจเลยว่าทำไมขายดี"], "last_styles": ["มุกตลก", "การเปรียบเทียบ (BAB)", "มุกตลก", "การเปรียบเทียบ (BAB)", "คำถาม", "มุกตลก", "มุกตลก", "การบอกต่อเฉยๆ", "การบอกต่อเฉยๆ", "มุกตลก", "มุกตลก", "ประสบการณ์ส่วนตัว (PAS)", "การบอกต่อเฉยๆ", "การเปรียบเทียบ (BAB)", "มุกตลก", "ประสบการณ์ส่วนตัว (PAS)", "คำถาม", "การบอกต่อเฉยๆ", "การเปรียบเทียบ (BAB)", "คำถาม", "คำถาม", "ประสบการณ์ส่วนตัว (PAS)", "คำถาม", "คำถาม", "การเปรียบเทียบ (BAB)", "มุกตลก", "คำถาม", "คำถาม", "มุกตลก", "การบอกต่อเฉยๆ", "ประสบการณ์ส่วนตัว (PAS)", "การบอกต่อเฉยๆ", "การเปรียบเทียบ (BAB)", "คำถาม", "มุกตลก", "การบอกต่อเฉยๆ", "มุกตลก", "การเปรียบเทียบ (BAB)", "มุกตลก", "ประสบการณ์ส่วนตัว (PAS)", "การเปรียบเทียบ (BAB)", "การเปรียบเทียบ (BAB)", "ประสบการณ์ส่วนตัว (PAS)", "คำถาม", "การบอกต่อเฉยๆ", "มุกตลก", "คำถาม", "มุกตลก", "คำถาม", "การบอกต่อเฉยๆ"], "last_roles": ["R7", "R4", "R2", "R2", "R6", "R4", "R1", "R3", "R4", "R3", "R8", "R2", "R1", "R4", "R6", "R1", "R4", "R2", "R8", "R2", "R5", "R7", "R2", "R5", "R5", "R7", "R3", "R7", "R1", "R8", "R3", "R7", "R7", "R8", "R1", "R4", "R3", "R3", "R2", "R1", "R5", "R6", "R4", "R6", "R6", "R4", "R5", "R1", "R2", "R7"], "recent_captions": ["เห็นคนพูดถึงเยอะเลยลอง ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Prowild โปรไวลด์ ซีเล็คเต็ด อาหารสุนัขทุกสายพ ราคาแค่ 1590 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "มีใครเป็นเหมือนผมไหม แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ เทียบกับ สินค้า แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น บ้านน็อคดาวน์ทรงโมเดิร์น ราคา . บาท ราคาแค่ 65000 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "อันนี้เกินคาดจริงๆ สินค้าตัวนี้เลยฮะ สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ ยกลัง Me o delite ราคาแค่ 1109 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เมื่อวานเพิ่งเจอ... สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น Prama อาหารสุนัขพราม่าเกรด Holistic มีให้เลือ ราคาแค่ 1250 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ตอนแรกไม่ได้จะซื้อ หลังเวทเสร็จเหนื่อยๆ ขี้เกียจเคี้ยวอกไก่ ได้ตัวนี้ดื่มทดแทนสะดวกมาก มีใครเคยลอง สินค้า ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น บ้านน็อคดาวน์ สำเร็จรูป ราคา . ราคาแค่ 150000 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "กำลังหาของแบบนี้อยู่พอดี ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Doge&amp;Orange ถุงมือเช็ดตัวสัตว์เลี้ยง ถุงมืออา ราคาแค่ 69 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "แชร์เผื่อมีคนกำลังหาอยู่ ของกินตัวนี้เลยฮะ ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ อ่างปลา บ่อบัว ขนาดใหญ่ // ราคาแค่ 2444 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "โดนป้ายยามาอีกที ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ PANDO Pet Dryer Room ราคาแค่ 9990 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ไม่คิดว่าจะ... แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ Petoya คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุน ราคาแค่ 490 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ลองแล้วเข้าใจเลยว่าทำไมขายดี ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ yoyopet : แปรงกําจัดขนสองด้าน แปรงสางขนเสีย ราคาแค่ 58 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เห็นคนพูดถึงเยอะเลยลอง ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ สายช้อปของคุ้มหารเฉลี่ยราคาต่อชิ้นแล้วประหยัดมาก คุ้มค่าน้ำตาไหล ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Pawdy อาหารสุนัขเกรดพรีเมียม สำหรับสุนัขสูงวั ราคาแค่ 643 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "มีใครเป็นเหมือนผมไหม สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ ลองซื้อ สินค้า ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง Rojeco เครื ่ องป ราคาแค่ 960 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "อันนี้เกินคาดจริงๆ ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก แวะมาแชร์ สินค้า ดีๆฮะ ตัวนี้มีจุดเด่นคือ สมาร์ทฮาร์ท โกลด์ ซีเลกต์ มูสลี่ ราคาแค่ 215 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เมื่อวานเพิ่งเจอ... แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น KUMAま ห้องน้ำแมว Minimal Design ราคาแค่ 1050 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ตอนแรกไม่ได้จะซื้อ ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ หลังเวทเสร็จเหนื่อยๆ ขี้เกียจเคี้ยวอกไก่ ได้ตัวนี้ดื่มทดแทนสะดวกมาก ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ เสื้อจุดให้สัตว์เลี้ยง เสื้อแมว เสื้อผ้าสัตว์ ราคาแค่ 51 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "กำลังหาของแบบนี้อยู่พอดี ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก ลองซื้อ ของใช้สัตว์เลี้ยง ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง ใส่โค้ดลดเพิ่ม Petology ทรายแมวภูเขาไฟ เก็บกล ราคาแค่ 510 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "แชร์เผื่อมีคนกำลังหาอยู่ แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น PANDO Double-Layer Pet Trolley ราคาแค่ 5990 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "โดนป้ายยามาอีกที สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ คอลลาเจนญี่ปุ่นบำรุงขนและข้อสำหรับสุนัขแมว สู ราคาแค่ 456 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ไม่คิดว่าจะ... สายช้อปของคุ้มหารเฉลี่ยราคาต่อชิ้นแล้วประหยัดมาก คุ้มค่าน้ำตาไหล เทียบกับ สินค้า แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น Doctor By BREATH CARE ราคาแค่ 1126 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ลองแล้วเข้าใจเลยว่าทำไมขายดี สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น ใส่โค้ดลดเพิ่ม Petology ห้องน้ำแมวอัตโนมัติ ด ราคาแค่ 13900 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เห็นคนพูดถึงเยอะเลยลอง เด็กๆ ที่บ้านชอบกันใหญ่ แย่งกันกินตึม สรรหามานานในที่สุดก็เจอ มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น โต๊ะวางชามอาหารน้องแมว และ น้องหมา น่ารัก ราคาแค่ 199 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "มีใครเป็นเหมือนผมไหม ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ ลองซื้อ ของใช้สัตว์เลี้ยง ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง ชุดสุดคุ้มFRONTLINE PLUS CAT ผลิตภัณฑ์หยดกำจั ราคาแค่ 982 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "อันนี้เกินคาดจริงๆ สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ มีใครเคยลอง ของกิน ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น ขนมแมวเลีย มีโอ ขนมแมวเลีย เพอร์เฟคมิกซ์ ราคาแค่ 760 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เมื่อวานเพิ่งเจอ... คนรักสัตว์อย่างเราหาของดีๆ มาให้เด็กๆ ตลอด ตัวนี้ตอบโจทย์มาก มีใครเคยลอง ของกิน ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น g x VetOLOGY ขนมเลียสำหรับแมวและสุนัข ราคาแค่ 368 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ตอนแรกไม่ได้จะซื้อ เด็กๆ ที่บ้านชอบกันใหญ่ แย่งกันกินตึม สรรหามานานในที่สุดก็เจอ เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น I&amp;CATอพาร์ทเมนท์แมว ผ้ากำมะหยี่ ชั้น ลับเล็บ ราคาแค่ 299 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "กำลังหาของแบบนี้อยู่พอดี ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Cutepol ทรายแมวเต้าหู้ ดับกลิ่นสูงสุด จับตัวก ราคาแค่ 499 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "แชร์เผื่อมีคนกำลังหาอยู่ ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น 🏆Pupping Petmat รุ่น Rug ราคาแค่ 4250 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "โดนป้ายยามาอีกที ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น สมาร์ทฮาร์ท อาหารสุนัข สำหรับลูกสุนัข รสเนื้อ ราคาแค่ 1030 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ไม่คิดว่าจะ... ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Pawdy อาหารสุนัขเกรดพรีเมียม Holistic สำหรับส ราคาแค่ 1359 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ลองแล้วเข้าใจเลยว่าทำไมขายดี สายช้อปของคุ้มหารเฉลี่ยราคาต่อชิ้นแล้วประหยัดมาก คุ้มค่าน้ำตาไหล แวะมาแชร์ สินค้า ดีๆฮะ ตัวนี้มีจุดเด่นคือ Virbac น้ำยาทำความสะอาดช่องหู อิพิโอติก EpiOt ราคาแค่ 493 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เห็นคนพูดถึงเยอะเลยลอง ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง ลองซื้อ ของกิน ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง แพ็ค CATE เคท ขนมแมวเลีย ราคาแค่ 639 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "มีใครเป็นเหมือนผมไหม ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ FABLEME —PET BASKET เข่งใส่แมว ราคาแค่ 200 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "อันนี้เกินคาดจริงๆ ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น สินค้าใหม่ PANDO Pet Hair ราคาแค่ 581 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เมื่อวานเพิ่งเจอ... สายช้อปของคุ้มหารเฉลี่ยราคาต่อชิ้นแล้วประหยัดมาก คุ้มค่าน้ำตาไหล มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น ทรายแมว แคสตี้ Kasty ทรายแมวเต้าหู้ ราคาแค่ 230 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ตอนแรกไม่ได้จะซื้อ สินค้าตัวนี้เลยฮะ ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ 😺 สินค้าอยู่ในไทย พร้อมส่ง 🐱 ราคาแค่ 1698 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "กำลังหาของแบบนี้อยู่พอดี แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ คละรสไม่ได้ สมาร์ทฮาร์ท อาหารสุนัขกระป๋อง กระ ราคาแค่ 1090 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "แชร์เผื่อมีคนกำลังหาอยู่ ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรั ราคาแค่ 8800 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "โดนป้ายยามาอีกที ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ ลดขนร่วง  ราคาแค่ 547 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ไม่คิดว่าจะ... ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ PET RECORDกระบะทรายแมวขนาดใหญ่ ขอบสูง ป้องกัน ราคาแค่ 52 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ลองแล้วเข้าใจเลยว่าทำไมขายดี ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก ลองซื้อ ของใช้สัตว์เลี้ยง ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง 🐈🐱Neakasa ห้องน้ำแมวอัตโนมัติ I Smart ราคาแค่ 10499 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เห็นคนพูดถึงเยอะเลยลอง คนรักสัตว์อย่างเราหาของดีๆ มาให้เด็กๆ ตลอด ตัวนี้ตอบโจทย์มาก เทียบกับ สินค้า แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น ชิ้นในแพ็คเกจใหญ่📍 ลูกกลิ้งกำจัดขน เก็บขนและฝ ราคาแค่ 60 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "มีใครเป็นเหมือนผมไหม หลังเวทเสร็จเหนื่อยๆ ขี้เกียจเคี้ยวอกไก่ ได้ตัวนี้ดื่มทดแทนสะดวกมาก เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น F&amp;G วิลล่าแมว Cat Villa ราคาแค่ 1999 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "อันนี้เกินคาดจริงๆ แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ ลองซื้อ ของใช้สัตว์เลี้ยง ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง แถมฝาปิด ส่งฟรี❤️ โอ่งแมวดินเผา16 นิ้ว ราคาแค่ 692 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เมื่อวานเพิ่งเจอ... หลังเวทเสร็จเหนื่อยๆ ขี้เกียจเคี้ยวอกไก่ ได้ตัวนี้ดื่มทดแทนสะดวกมาก มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น คอนโดแมว คอนโดแมวไม้ บ้านแมว เหมาะสำหรับเลี้ย ราคาแค่ 658 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ตอนแรกไม่ได้จะซื้อ หลังเวทเสร็จเหนื่อยๆ ขี้เกียจเคี้ยวอกไก่ ได้ตัวนี้ดื่มทดแทนสะดวกมาก แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ Petoya คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุน ราคาแค่ 490 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "กำลังหาของแบบนี้อยู่พอดี ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Dog Days อาหารลูกสุนัข สูตร ราคาแค่ 690 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "แชร์เผื่อมีคนกำลังหาอยู่ เด็กๆ ที่บ้านชอบกันใหญ่ แย่งกันกินตึม สรรหามานานในที่สุดก็เจอ มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น ยกโหล Nekko อาหารเปียกแมว กรัม12ซอง ราคาแค่ 159 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇\n🔥 โปรโมชั่น: ฿159", "โดนป้ายยามาอีกที ตอนแรกผมก็นึกว่า ตะกร้าที่นอนแมว รุ่น Fableme ทรงเข่งมินิมอล ราคา 220 บาทอันนี้ จะกลายเป็นที่เก็บกระดูกของน้องตูบซะแล้วเพราะหน้าตาคล้ายเข่งปลาทูแถวบ้านเหลือเกิน แต่พอสอยมาลอง เจ้านายกลับเข้าไปนอนขดสิงสถิตยาวไม่ยอมลุกเลยโฮ่ง ใครกำลังหา ที่นอนแมวราคาประหยัด ไปแต่งบ้านสวยๆ แชร์ต่อให้เพื่อนที่เจอปัญหาซื้อเตียงแพงแล้วแมวนอนกล่องกระดาษเซฟเก็บไว้ดูเลยฮะ กดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇\n🔥 โปรโมชั่น: ฿220", "ไม่คิดว่าจะเจอปัญหากลิ่นตัวแรงจนมนุษย์แม่ส่ายหัว แถมขนยังแห้งฟูจนหมดหล่อ มีบ้านไหนกำลังมองหาวิธีดับกลิ่นตัวสุนัขแบบเร่งด่วนบ้างไหมฮะ? แต่พอผมได้สเปรย์สัตว์เลี้ยงขวดนี้ราคาแค่ 210 บาท มาฉีดปุ๊บก็ช่วยดับกลิ่นสาบได้ทันที แถมยังช่วยบำรุงขนของน้องตูบให้นุ่มสลวยน่ากอดขึ้นเยอะเลยโฮ่ง เซฟเก็บไว้ดูตอนช้อปหรือแชร์ต่อให้เพื่อนที่เจอปัญหานี้ด่วนๆ เลยฮะ กดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇\n🔥 โปรโมชั่น: ฿210", "ลองแล้วเข้าใจเลยว่าทำไมขายดี ผมเห็นแม่กังวลเรื่องคราบน้ำตากับขนที่ร่วงเต็มบ้าน เลยได้ลองอาหารสุนัขรสแกะถุงนี้ฮะ ตัวนี้ช่วยลดคราบน้ำตาสุนัขและยังเป็นสูตรที่ช่วยลดขนร่วงด้วย ในราคา 542 บาทเองฮะ บ้านไหนที่เจอปัญหานี้เหมือนกันเซฟโพสต์นี้เก็บไว้ไปลองดูนะโฮ่ง กดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇\n🔥 โปรโมชั่น: ฿542"]}</t>
+          <t>{"last_personas": ["C", "G", "F", "E", "C", "H", "C", "G", "F", "A", "G", "E", "C", "C", "H", "E", "D", "C", "H", "F", "E", "F", "B", "E", "E", "F", "B", "E", "H", "D", "C", "H", "G", "G", "D", "A", "F", "H", "F", "G", "D", "A", "G", "A", "F", "F", "A", "H", "F", "G"], "last_hooks": ["ไม่คิดว่าจะ...", "ลองแล้วเข้าใจเลยว่าทำไมขายดี", "เห็นคนพูดถึงเยอะเลยลอง", "มีใครเป็นเหมือนผมไหม", "อันนี้เกินคาดจริงๆ", "เมื่อวานเพิ่งเจอ...", "ตอนแรกไม่ได้จะซื้อ", "กำลังหาของแบบนี้อยู่พอดี", "แชร์เผื่อมีคนกำลังหาอยู่", "โดนป้ายยามาอีกที", "ไม่คิดว่าจะ...", "ลองแล้วเข้าใจเลยว่าทำไมขายดี", "เห็นคนพูดถึงเยอะเลยลอง", "มีใครเป็นเหมือนผมไหม", "อันนี้เกินคาดจริงๆ", "เมื่อวานเพิ่งเจอ...", "ตอนแรกไม่ได้จะซื้อ", "กำลังหาของแบบนี้อยู่พอดี", "แชร์เผื่อมีคนกำลังหาอยู่", "โดนป้ายยามาอีกที", "ไม่คิดว่าจะ...", "ลองแล้วเข้าใจเลยว่าทำไมขายดี", "เห็นคนพูดถึงเยอะเลยลอง", "มีใครเป็นเหมือนผมไหม", "อันนี้เกินคาดจริงๆ", "เมื่อวานเพิ่งเจอ...", "ตอนแรกไม่ได้จะซื้อ", "กำลังหาของแบบนี้อยู่พอดี", "แชร์เผื่อมีคนกำลังหาอยู่", "โดนป้ายยามาอีกที", "ไม่คิดว่าจะ...", "ลองแล้วเข้าใจเลยว่าทำไมขายดี", "เห็นคนพูดถึงเยอะเลยลอง", "มีใครเป็นเหมือนผมไหม", "อันนี้เกินคาดจริงๆ", "เมื่อวานเพิ่งเจอ...", "ตอนแรกไม่ได้จะซื้อ", "กำลังหาของแบบนี้อยู่พอดี", "แชร์เผื่อมีคนกำลังหาอยู่", "โดนป้ายยามาอีกที", "ไม่คิดว่าจะ...", "ลองแล้วเข้าใจเลยว่าทำไมขายดี", "เห็นคนพูดถึงเยอะเลยลอง", "มีใครเป็นเหมือนผมไหม", "อันนี้เกินคาดจริงๆ", "เมื่อวานเพิ่งเจอ...", "ตอนแรกไม่ได้จะซื้อ", "กำลังหาของแบบนี้อยู่พอดี", "แชร์เผื่อมีคนกำลังหาอยู่", "โดนป้ายยามาอีกที"], "last_styles": ["คำถาม", "คำถาม", "มุกตลก", "การเปรียบเทียบ (BAB)", "มุกตลก", "การเปรียบเทียบ (BAB)", "คำถาม", "มุกตลก", "มุกตลก", "การบอกต่อเฉยๆ", "การบอกต่อเฉยๆ", "มุกตลก", "มุกตลก", "ประสบการณ์ส่วนตัว (PAS)", "การบอกต่อเฉยๆ", "การเปรียบเทียบ (BAB)", "มุกตลก", "ประสบการณ์ส่วนตัว (PAS)", "คำถาม", "การบอกต่อเฉยๆ", "การเปรียบเทียบ (BAB)", "คำถาม", "คำถาม", "ประสบการณ์ส่วนตัว (PAS)", "คำถาม", "คำถาม", "การเปรียบเทียบ (BAB)", "มุกตลก", "คำถาม", "คำถาม", "มุกตลก", "การบอกต่อเฉยๆ", "ประสบการณ์ส่วนตัว (PAS)", "การบอกต่อเฉยๆ", "การเปรียบเทียบ (BAB)", "คำถาม", "มุกตลก", "การบอกต่อเฉยๆ", "มุกตลก", "การเปรียบเทียบ (BAB)", "มุกตลก", "ประสบการณ์ส่วนตัว (PAS)", "การเปรียบเทียบ (BAB)", "การเปรียบเทียบ (BAB)", "ประสบการณ์ส่วนตัว (PAS)", "คำถาม", "การบอกต่อเฉยๆ", "มุกตลก", "คำถาม", "มุกตลก"], "last_roles": ["R1", "R3", "R7", "R4", "R2", "R2", "R6", "R4", "R1", "R3", "R4", "R3", "R8", "R2", "R1", "R4", "R6", "R1", "R4", "R2", "R8", "R2", "R5", "R7", "R2", "R5", "R5", "R7", "R3", "R7", "R1", "R8", "R3", "R7", "R7", "R8", "R1", "R4", "R3", "R3", "R2", "R1", "R5", "R6", "R4", "R6", "R6", "R4", "R5", "R1"], "recent_captions": ["ไม่คิดว่าจะ... ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น MOMOVIDA CC- กระบะทรายแมวขนาดใหญ่ ห้องน้ำแมวข ราคาแค่ 639 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ลองแล้วเข้าใจเลยว่าทำไมขายดี ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น ไดร์เป่าขนสุนัข ขนแมว ขนหมา เครื่องเป่าขนสุนั ราคาแค่ 2989 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เห็นคนพูดถึงเยอะเลยลอง ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Prowild โปรไวลด์ ซีเล็คเต็ด อาหารสุนัขทุกสายพ ราคาแค่ 1590 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "มีใครเป็นเหมือนผมไหม แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ เทียบกับ สินค้า แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น บ้านน็อคดาวน์ทรงโมเดิร์น ราคา . บาท ราคาแค่ 65000 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "อันนี้เกินคาดจริงๆ สินค้าตัวนี้เลยฮะ สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ ยกลัง Me o delite ราคาแค่ 1109 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เมื่อวานเพิ่งเจอ... สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น Prama อาหารสุนัขพราม่าเกรด Holistic มีให้เลือ ราคาแค่ 1250 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ตอนแรกไม่ได้จะซื้อ หลังเวทเสร็จเหนื่อยๆ ขี้เกียจเคี้ยวอกไก่ ได้ตัวนี้ดื่มทดแทนสะดวกมาก มีใครเคยลอง สินค้า ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น บ้านน็อคดาวน์ สำเร็จรูป ราคา . ราคาแค่ 150000 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "กำลังหาของแบบนี้อยู่พอดี ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Doge&amp;Orange ถุงมือเช็ดตัวสัตว์เลี้ยง ถุงมืออา ราคาแค่ 69 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "แชร์เผื่อมีคนกำลังหาอยู่ ของกินตัวนี้เลยฮะ ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ อ่างปลา บ่อบัว ขนาดใหญ่ // ราคาแค่ 2444 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "โดนป้ายยามาอีกที ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ PANDO Pet Dryer Room ราคาแค่ 9990 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ไม่คิดว่าจะ... แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ Petoya คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุน ราคาแค่ 490 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ลองแล้วเข้าใจเลยว่าทำไมขายดี ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ yoyopet : แปรงกําจัดขนสองด้าน แปรงสางขนเสีย ราคาแค่ 58 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เห็นคนพูดถึงเยอะเลยลอง ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ สายช้อปของคุ้มหารเฉลี่ยราคาต่อชิ้นแล้วประหยัดมาก คุ้มค่าน้ำตาไหล ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Pawdy อาหารสุนัขเกรดพรีเมียม สำหรับสุนัขสูงวั ราคาแค่ 643 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "มีใครเป็นเหมือนผมไหม สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ ลองซื้อ สินค้า ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง Rojeco เครื ่ องป ราคาแค่ 960 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "อันนี้เกินคาดจริงๆ ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก แวะมาแชร์ สินค้า ดีๆฮะ ตัวนี้มีจุดเด่นคือ สมาร์ทฮาร์ท โกลด์ ซีเลกต์ มูสลี่ ราคาแค่ 215 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เมื่อวานเพิ่งเจอ... แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น KUMAま ห้องน้ำแมว Minimal Design ราคาแค่ 1050 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ตอนแรกไม่ได้จะซื้อ ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ หลังเวทเสร็จเหนื่อยๆ ขี้เกียจเคี้ยวอกไก่ ได้ตัวนี้ดื่มทดแทนสะดวกมาก ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ เสื้อจุดให้สัตว์เลี้ยง เสื้อแมว เสื้อผ้าสัตว์ ราคาแค่ 51 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "กำลังหาของแบบนี้อยู่พอดี ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก ลองซื้อ ของใช้สัตว์เลี้ยง ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง ใส่โค้ดลดเพิ่ม Petology ทรายแมวภูเขาไฟ เก็บกล ราคาแค่ 510 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "แชร์เผื่อมีคนกำลังหาอยู่ แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น PANDO Double-Layer Pet Trolley ราคาแค่ 5990 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "โดนป้ายยามาอีกที สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ คอลลาเจนญี่ปุ่นบำรุงขนและข้อสำหรับสุนัขแมว สู ราคาแค่ 456 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ไม่คิดว่าจะ... สายช้อปของคุ้มหารเฉลี่ยราคาต่อชิ้นแล้วประหยัดมาก คุ้มค่าน้ำตาไหล เทียบกับ สินค้า แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น Doctor By BREATH CARE ราคาแค่ 1126 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ลองแล้วเข้าใจเลยว่าทำไมขายดี สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น ใส่โค้ดลดเพิ่ม Petology ห้องน้ำแมวอัตโนมัติ ด ราคาแค่ 13900 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เห็นคนพูดถึงเยอะเลยลอง เด็กๆ ที่บ้านชอบกันใหญ่ แย่งกันกินตึม สรรหามานานในที่สุดก็เจอ มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น โต๊ะวางชามอาหารน้องแมว และ น้องหมา น่ารัก ราคาแค่ 199 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "มีใครเป็นเหมือนผมไหม ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ ลองซื้อ ของใช้สัตว์เลี้ยง ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง ชุดสุดคุ้มFRONTLINE PLUS CAT ผลิตภัณฑ์หยดกำจั ราคาแค่ 982 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "อันนี้เกินคาดจริงๆ สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ มีใครเคยลอง ของกิน ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น ขนมแมวเลีย มีโอ ขนมแมวเลีย เพอร์เฟคมิกซ์ ราคาแค่ 760 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เมื่อวานเพิ่งเจอ... คนรักสัตว์อย่างเราหาของดีๆ มาให้เด็กๆ ตลอด ตัวนี้ตอบโจทย์มาก มีใครเคยลอง ของกิน ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น g x VetOLOGY ขนมเลียสำหรับแมวและสุนัข ราคาแค่ 368 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ตอนแรกไม่ได้จะซื้อ เด็กๆ ที่บ้านชอบกันใหญ่ แย่งกันกินตึม สรรหามานานในที่สุดก็เจอ เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น I&amp;CATอพาร์ทเมนท์แมว ผ้ากำมะหยี่ ชั้น ลับเล็บ ราคาแค่ 299 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "กำลังหาของแบบนี้อยู่พอดี ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Cutepol ทรายแมวเต้าหู้ ดับกลิ่นสูงสุด จับตัวก ราคาแค่ 499 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "แชร์เผื่อมีคนกำลังหาอยู่ ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น 🏆Pupping Petmat รุ่น Rug ราคาแค่ 4250 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "โดนป้ายยามาอีกที ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น สมาร์ทฮาร์ท อาหารสุนัข สำหรับลูกสุนัข รสเนื้อ ราคาแค่ 1030 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ไม่คิดว่าจะ... ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Pawdy อาหารสุนัขเกรดพรีเมียม Holistic สำหรับส ราคาแค่ 1359 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ลองแล้วเข้าใจเลยว่าทำไมขายดี สายช้อปของคุ้มหารเฉลี่ยราคาต่อชิ้นแล้วประหยัดมาก คุ้มค่าน้ำตาไหล แวะมาแชร์ สินค้า ดีๆฮะ ตัวนี้มีจุดเด่นคือ Virbac น้ำยาทำความสะอาดช่องหู อิพิโอติก EpiOt ราคาแค่ 493 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เห็นคนพูดถึงเยอะเลยลอง ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง ลองซื้อ ของกิน ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง แพ็ค CATE เคท ขนมแมวเลีย ราคาแค่ 639 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "มีใครเป็นเหมือนผมไหม ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ FABLEME —PET BASKET เข่งใส่แมว ราคาแค่ 200 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "อันนี้เกินคาดจริงๆ ในฐานะแม่บ้านที่ชอบหาของเข้าครัว ดูแลคนในบ้าน แนะนำเลยค่ะ เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น สินค้าใหม่ PANDO Pet Hair ราคาแค่ 581 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เมื่อวานเพิ่งเจอ... สายช้อปของคุ้มหารเฉลี่ยราคาต่อชิ้นแล้วประหยัดมาก คุ้มค่าน้ำตาไหล มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น ทรายแมว แคสตี้ Kasty ทรายแมวเต้าหู้ ราคาแค่ 230 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ตอนแรกไม่ได้จะซื้อ สินค้าตัวนี้เลยฮะ ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ 😺 สินค้าอยู่ในไทย พร้อมส่ง 🐱 ราคาแค่ 1698 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "กำลังหาของแบบนี้อยู่พอดี แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ คละรสไม่ได้ สมาร์ทฮาร์ท อาหารสุนัขกระป๋อง กระ ราคาแค่ 1090 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "แชร์เผื่อมีคนกำลังหาอยู่ ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรั ราคาแค่ 8800 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "โดนป้ายยามาอีกที ช่วงควบคุมอาหาร ดูแลหุ่นอยู่ ได้ตัวนี้ช่วยชีวิตไว้เลย แคลน้อยโปรตีนสูง เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ ลดขนร่วง  ราคาแค่ 547 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ไม่คิดว่าจะ... ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ สายของอร่อยอย่างเราลองแล้วดื่มด่ำมาก ฟินสุดๆ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ PET RECORDกระบะทรายแมวขนาดใหญ่ ขอบสูง ป้องกัน ราคาแค่ 52 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ลองแล้วเข้าใจเลยว่าทำไมขายดี ในฐานะพ่อบ้านที่ชอบจัดบ้านดูแลงานบ้าน บอกเลยว่าถูกใจมาก ลองซื้อ ของใช้สัตว์เลี้ยง ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง 🐈🐱Neakasa ห้องน้ำแมวอัตโนมัติ I Smart ราคาแค่ 10499 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เห็นคนพูดถึงเยอะเลยลอง คนรักสัตว์อย่างเราหาของดีๆ มาให้เด็กๆ ตลอด ตัวนี้ตอบโจทย์มาก เทียบกับ สินค้า แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น ชิ้นในแพ็คเกจใหญ่📍 ลูกกลิ้งกำจัดขน เก็บขนและฝ ราคาแค่ 60 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "มีใครเป็นเหมือนผมไหม หลังเวทเสร็จเหนื่อยๆ ขี้เกียจเคี้ยวอกไก่ ได้ตัวนี้ดื่มทดแทนสะดวกมาก เทียบกับ ของใช้สัตว์เลี้ยง แบบเดิมๆ ที่เคยใช้ ตัวนี้คือจุดเด่น F&amp;G วิลล่าแมว Cat Villa ราคาแค่ 1999 บาท ดีกว่าเห็นๆ เลยฮะ\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "อันนี้เกินคาดจริงๆ แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ ลองซื้อ ของใช้สัตว์เลี้ยง ตัวนี้มาใช้ได้สักพักแล้วฮะ รู้สึกสะดวกสบายขึ้นเยอะ โดยเฉพาะเรื่อง แถมฝาปิด ส่งฟรี❤️ โอ่งแมวดินเผา16 นิ้ว ราคาแค่ 692 บาท ดีจริง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "เมื่อวานเพิ่งเจอ... หลังเวทเสร็จเหนื่อยๆ ขี้เกียจเคี้ยวอกไก่ ได้ตัวนี้ดื่มทดแทนสะดวกมาก มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น คอนโดแมว คอนโดแมวไม้ บ้านแมว เหมาะสำหรับเลี้ย ราคาแค่ 658 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "ตอนแรกไม่ได้จะซื้อ หลังเวทเสร็จเหนื่อยๆ ขี้เกียจเคี้ยวอกไก่ ได้ตัวนี้ดื่มทดแทนสะดวกมาก แวะมาแชร์ ของใช้สัตว์เลี้ยง ดีๆฮะ ตัวนี้มีจุดเด่นคือ Petoya คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุน ราคาแค่ 490 บาท เผื่อใครกำลังสนใจอยู่\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "กำลังหาของแบบนี้อยู่พอดี ของใช้สัตว์เลี้ยงตัวนี้เลยฮะ แช่ตู้เย็นที่ออฟฟิศไว้ เวลาหิวดึกหิวยามบ่ายช่วยชีวิตพนักงานออฟฟิศได้เยอะ ตอนแรกกังวลว่าจะไม่โอเค แต่พอลองแล้วชอบเลย รอดตายแล้วเรา 555 จุดเด่นคือ Dog Days อาหารลูกสุนัข สูตร ราคาแค่ 690 บาท\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇", "แชร์เผื่อมีคนกำลังหาอยู่ เด็กๆ ที่บ้านชอบกันใหญ่ แย่งกันกินตึม สรรหามานานในที่สุดก็เจอ มีใครเคยลอง ของใช้สัตว์เลี้ยง ตัวนี้รึยังฮะ ส่วนตัวประทับใจจุดเด่น ยกโหล Nekko อาหารเปียกแมว กรัม12ซอง ราคาแค่ 159 บาท คิดว่าไงกันบ้าง\n\nกดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇\n🔥 โปรโมชั่น: ฿159", "โดนป้ายยามาอีกที ตอนแรกผมก็นึกว่า ตะกร้าที่นอนแมว รุ่น Fableme ทรงเข่งมินิมอล ราคา 220 บาทอันนี้ จะกลายเป็นที่เก็บกระดูกของน้องตูบซะแล้วเพราะหน้าตาคล้ายเข่งปลาทูแถวบ้านเหลือเกิน แต่พอสอยมาลอง เจ้านายกลับเข้าไปนอนขดสิงสถิตยาวไม่ยอมลุกเลยโฮ่ง ใครกำลังหา ที่นอนแมวราคาประหยัด ไปแต่งบ้านสวยๆ แชร์ต่อให้เพื่อนที่เจอปัญหาซื้อเตียงแพงแล้วแมวนอนกล่องกระดาษเซฟเก็บไว้ดูเลยฮะ กดลิ้งในคอมเมนต์แรกได้เลยฮะ 👇\n🔥 โปรโมชั่น: ฿220"]}</t>
         </is>
       </c>
     </row>

</xml_diff>